<commit_message>
Add Kanata, Discovery and Fermeuse; drop electrification assumption; rerun
Register:
- Add Kanata LNG (12.0 mtpa) and Discovery LNG (20.0 mtpa) as early_proposed
- Give Fermeuse a derived capacity of 5.0 mtpa, constrained by the stated
  9.7 Tcf Jeanne d'Arc reserve over a 40-year life
- Record regulator and proponent sources confirming Grassy Point, Bear Head
  and Goldboro are cancelled, since third-party lists show them as live

Method:
- Apply the gas turbine liquefaction factor of 0.29 to all terminals for their
  whole operating life. Electric drive is no longer assumed for any project.
  Only Cedar and Woodfibre have interconnection works under construction; the
  rest rest on MOUs or aspirations conditional on transmission that does not
  exist. Previous classifications retained in liquefaction_drive_note.

Results rerun across all scenarios, chains and groups.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Asset_Register.xlsx
+++ b/Inputs/Canada_LNG_Asset_Register.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -526,7 +526,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 13:20 UTC</t>
+          <t>2026-08-20 10:00 UTC</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>All Canadian LNG terminals in GEM GGIT (Sep 2025), plus three not in GEM found by research: Summit Lake PG LNG, Marinvest Baie-Comeau and the Tilbury Marine Jetty.</t>
+          <t>All Canadian LNG terminals in GEM GGIT (Sep 2025), plus projects not in GEM found by research: Summit Lake PG LNG, Marinvest Baie-Comeau, the Tilbury Marine Jetty, and Kanata LNG. Discovery LNG is in GEM but was moved from inactive to early_proposed pending verification.</t>
         </is>
       </c>
     </row>
@@ -985,6 +985,42 @@
       <c r="B53" s="4" t="inlineStr">
         <is>
           <t>69.78 bcm/y of live pipeline capacity against 62.65 of demand looks comfortable, but capacity is not fungible. Spare room on Prince Rupert Gas Transmission cannot serve Kitimat. Only the per-line check tells you anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Cancelled projects mislisted as live</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Several third-party summaries list Grassy Point, Bear Head and Goldboro as live proposals. Each is confirmed cancelled by a regulator or by the proponent, with the evidence recorded in the relevant row. Those summaries appear to rest on regulatory records from 2018 and 2019 without checking whether the assessments were subsequently terminated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Fermeuse capacity is derived</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Fermeuse Energy has not published a liquefaction capacity. The register records 5.0 mtpa, the lowest defensible derivation from the stated 9.7 Tcf Jeanne d'Arc reserve over a 40-year life. This is an exception to the nameplate convention and is flagged in capacity_basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Electrification is not assumed</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>liquefaction_drive is gas_turbine for every export and bunkering asset. Previous electric_committed / electric_planned / not_published classifications are retained in liquefaction_drive_note, prefixed with 'previously classified as'.</t>
         </is>
       </c>
     </row>
@@ -999,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB56"/>
+  <dimension ref="A1:BB57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1447,10 +1483,7 @@
       <c r="Z2" t="n">
         <v>3800</v>
       </c>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
       <c r="AC2" s="4" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
       <c r="AE2" s="4" t="inlineStr">
         <is>
           <t>JV partners lift their own equity share rather than contracting third-party offtake</t>
@@ -1461,7 +1494,6 @@
           <t>export</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="b">
         <v>0</v>
       </c>
@@ -1500,7 +1532,6 @@
           <t>Partial only - Phase 1 liquefaction runs on gas turbines</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="n">
         <v>40</v>
       </c>
@@ -1598,7 +1629,6 @@
           <t>Tilbury Island</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Fortis Inc [100.0%]</t>
@@ -1614,8 +1644,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>2018</v>
       </c>
@@ -1660,27 +1688,21 @@
           <t>Port of Vancouver ship-to-ship bunkering</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
       <c r="AC3" s="4" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
       <c r="AE3" s="4" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>not_published</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ3" s="4" t="inlineStr">
         <is>
-          <t>Drive type not published. These are small peak-shaving, off-grid or bunkering facilities, several predating 2000. The model applies liquefaction_drive_default from Parameters. Combined capacity is 1.22 mtpa against 45.4 mtpa of export, so the choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
+          <t>previously classified as not_published. Drive type not published. These are small peak-shaving, off-grid or bunkering facilities, several predating 2000. The model applies liquefaction_drive_default from Parameters. Combined capacity is 1.22 mtpa against 45.4 mtpa of export, so the choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -1696,15 +1718,11 @@
       <c r="AM3" s="4" t="inlineStr"/>
       <c r="AN3" s="4" t="inlineStr"/>
       <c r="AO3" s="4" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
       <c r="AS3" s="4" t="inlineStr">
         <is>
           <t>No licence identified</t>
         </is>
       </c>
-      <c r="AT3" t="inlineStr"/>
       <c r="AU3" t="inlineStr">
         <is>
           <t>T100000131044</t>
@@ -1749,8 +1767,6 @@
           <t>Energir LNG Facility (Montreal)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
           <t>operating</t>
@@ -1796,8 +1812,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>1976</v>
       </c>
@@ -1842,19 +1856,13 @@
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
       <c r="AC4" s="4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
       <c r="AE4" s="4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
           <t>storage and liquefaction</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr">
         <is>
           <t>not_published</t>
@@ -1878,16 +1886,11 @@
       <c r="AM4" s="4" t="inlineStr"/>
       <c r="AN4" s="4" t="inlineStr"/>
       <c r="AO4" s="4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
       <c r="AS4" s="4" t="inlineStr">
         <is>
           <t>No export licence - domestic facility</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
       <c r="AV4" s="4" t="inlineStr"/>
       <c r="AW4" s="4" t="inlineStr">
         <is>
@@ -1919,8 +1922,6 @@
           <t>Mt. Hayes LNG Facility</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
           <t>operating</t>
@@ -1966,8 +1967,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>2011</v>
       </c>
@@ -2012,19 +2011,13 @@
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
       <c r="AC5" s="4" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
       <c r="AE5" s="4" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
           <t>storage and liquefaction</t>
         </is>
       </c>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr">
         <is>
           <t>not_published</t>
@@ -2048,16 +2041,11 @@
       <c r="AM5" s="4" t="inlineStr"/>
       <c r="AN5" s="4" t="inlineStr"/>
       <c r="AO5" s="4" t="inlineStr"/>
-      <c r="AP5" t="inlineStr"/>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
       <c r="AS5" s="4" t="inlineStr">
         <is>
           <t>No export licence - domestic facility</t>
         </is>
       </c>
-      <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
       <c r="AV5" s="4" t="inlineStr"/>
       <c r="AW5" s="4" t="inlineStr">
         <is>
@@ -2124,7 +2112,6 @@
           <t>Tilbury Island</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Fortis Inc [100.0%]</t>
@@ -2140,8 +2127,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>1971</v>
       </c>
@@ -2186,19 +2171,13 @@
           <t>Not applicable - Lower Mainland gas system</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
       <c r="AC6" s="4" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
       <c r="AE6" s="4" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr">
         <is>
           <t>not_published</t>
@@ -2222,15 +2201,11 @@
       <c r="AM6" s="4" t="inlineStr"/>
       <c r="AN6" s="4" t="inlineStr"/>
       <c r="AO6" s="4" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
       <c r="AS6" s="4" t="inlineStr">
         <is>
           <t>NRCan lists this unit as a domestic liquefaction facility, not an export project</t>
         </is>
       </c>
-      <c r="AT6" t="inlineStr"/>
       <c r="AU6" t="inlineStr">
         <is>
           <t>T100000131044</t>
@@ -2279,8 +2254,6 @@
           <t>Tamaska LNG Facility (Fort Nelson)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
           <t>operating</t>
@@ -2326,8 +2299,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>2021</v>
       </c>
@@ -2372,19 +2343,13 @@
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
       <c r="AC7" s="4" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
       <c r="AE7" s="4" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
           <t>liquefaction</t>
         </is>
       </c>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr">
         <is>
           <t>not_published</t>
@@ -2408,16 +2373,11 @@
       <c r="AM7" s="4" t="inlineStr"/>
       <c r="AN7" s="4" t="inlineStr"/>
       <c r="AO7" s="4" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
       <c r="AS7" s="4" t="inlineStr">
         <is>
           <t>No export licence - domestic facility</t>
         </is>
       </c>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
       <c r="AV7" s="4" t="inlineStr"/>
       <c r="AW7" s="4" t="inlineStr">
         <is>
@@ -2449,8 +2409,6 @@
           <t>Port of Hamilton LNG Terminal</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>operating</t>
@@ -2496,15 +2454,11 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
       <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>Not applicable - domestic facility</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" s="4" t="inlineStr">
         <is>
           <t>Not available</t>
@@ -2538,19 +2492,13 @@
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
       <c r="AC8" s="4" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
       <c r="AE8" s="4" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
           <t>import</t>
         </is>
       </c>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr">
         <is>
           <t>not_published</t>
@@ -2574,16 +2522,11 @@
       <c r="AM8" s="4" t="inlineStr"/>
       <c r="AN8" s="4" t="inlineStr"/>
       <c r="AO8" s="4" t="inlineStr"/>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
       <c r="AS8" s="4" t="inlineStr">
         <is>
           <t>No export licence - domestic facility</t>
         </is>
       </c>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
       <c r="AV8" s="4" t="inlineStr"/>
       <c r="AW8" s="4" t="inlineStr">
         <is>
@@ -2615,8 +2558,6 @@
           <t>Cedar FLNG Terminal</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" s="7" t="inlineStr">
         <is>
           <t>under_construction</t>
@@ -2642,7 +2583,6 @@
           <t>Kitimat</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Haisla Nation [50.1%]; Pembina Pipeline Corp [49.9%] (via Cedar LNG Partners LP)</t>
@@ -2741,12 +2681,12 @@
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>electric_committed</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ9" s="4" t="inlineStr">
         <is>
-          <t>Designed for electric drive on BC Hydro renewable supply. Served by the North Coast transmission build-out.</t>
+          <t>previously classified as electric_committed. Designed for electric drive on BC Hydro renewable supply. Served by the North Coast transmission build-out.</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
@@ -2774,7 +2714,6 @@
           <t>Committed - design is electric drive</t>
         </is>
       </c>
-      <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="n">
         <v>40</v>
       </c>
@@ -2837,8 +2776,6 @@
           <t>Woodfibre LNG Terminal</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" s="7" t="inlineStr">
         <is>
           <t>under_construction</t>
@@ -2961,18 +2898,17 @@
           <t>export</t>
         </is>
       </c>
-      <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="b">
         <v>1</v>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>electric_committed</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ10" s="4" t="inlineStr">
         <is>
-          <t>Electric motors on BC Hydro supply. Interconnection works under construction, in service from October 2026.</t>
+          <t>previously classified as electric_committed. Electric motors on BC Hydro supply. Interconnection works under construction, in service from October 2026.</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr">
@@ -3000,7 +2936,6 @@
           <t>Committed - interconnection under construction</t>
         </is>
       </c>
-      <c r="AP10" t="inlineStr"/>
       <c r="AQ10" t="n">
         <v>40</v>
       </c>
@@ -3125,7 +3060,6 @@
       <c r="N11" t="b">
         <v>0</v>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>2030</v>
       </c>
@@ -3169,28 +3103,24 @@
       <c r="Z11" t="n">
         <v>3800</v>
       </c>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
       <c r="AC11" s="4" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
       <c r="AE11" s="4" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="b">
         <v>1</v>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>electric_planned</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ11" s="4" t="inlineStr">
         <is>
-          <t>Proponent states a transition to electric motors as more renewable power becomes available. No firm date or contracted supply.</t>
+          <t>previously classified as electric_planned. Proponent states a transition to electric motors as more renewable power becomes available. No firm date or contracted supply.</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
@@ -3218,7 +3148,6 @@
           <t>Aspirational - conditional on power availability, no firm date</t>
         </is>
       </c>
-      <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="n">
         <v>40</v>
       </c>
@@ -3285,8 +3214,6 @@
           <t>Ksi Lisims FLNG Terminal</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
           <t>advanced_proposed</t>
@@ -3312,7 +3239,6 @@
           <t>Gingolx</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr">
         <is>
           <t>TotalEnergies SE [5.0%]; Nisga'a Nation; Rockies LNG; Western LNG LLC</t>
@@ -3331,7 +3257,6 @@
       <c r="N12" t="b">
         <v>0</v>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>2029</v>
       </c>
@@ -3407,12 +3332,12 @@
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>electric_planned</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ12" s="4" t="inlineStr">
         <is>
-          <t>MOU with BC Hydro signed January 2026 for up to 600 MW, conditional on the North Coast Transmission Line expansion. Permits require net-zero ready by 2030. An MOU is not a firm supply agreement.</t>
+          <t>previously classified as electric_planned. MOU with BC Hydro signed January 2026 for up to 600 MW, conditional on the North Coast Transmission Line expansion. Permits require net-zero ready by 2030. An MOU is not a firm supply agreement.</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
@@ -3440,7 +3365,6 @@
           <t>Contractual condition - permits require net-zero ready by 2030; MOU not yet a firm supply agreement</t>
         </is>
       </c>
-      <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="n">
         <v>40</v>
       </c>
@@ -3542,7 +3466,6 @@
           <t>Tilbury Island</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Fortis Inc [100.0%]</t>
@@ -3561,8 +3484,6 @@
       <c r="N13" t="b">
         <v>0</v>
       </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
       <c r="Q13" s="4" t="inlineStr">
         <is>
           <t>CER export licence, 25 year term</t>
@@ -3586,7 +3507,6 @@
           <t>Two components: a storage tank providing backup energy supply to the Lower Mainland, and additional liquefaction. FortisBC frames it as Lower Mainland resiliency plus emerging marine fuelling markets. NRCan nonetheless lists Phase 2 as an export project holding a 25 year licence.</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
       <c r="W13" s="4" t="inlineStr">
         <is>
           <t>Mixed. One component is a storage tank providing Lower Mainland backup supply, which is domestic; the other is liquefaction serving marine fuelling. FortisBC does not publish the split.</t>
@@ -3602,27 +3522,21 @@
           <t>Lower Mainland supply and Port of Vancouver bunkering</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
       <c r="AC13" s="4" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
       <c r="AE13" s="4" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>not_published</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ13" s="4" t="inlineStr">
         <is>
-          <t>Drive type not published. These are small peak-shaving, off-grid or bunkering facilities, several predating 2000. The model applies liquefaction_drive_default from Parameters. Combined capacity is 1.22 mtpa against 45.4 mtpa of export, so the choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
+          <t>previously classified as not_published. Drive type not published. These are small peak-shaving, off-grid or bunkering facilities, several predating 2000. The model applies liquefaction_drive_default from Parameters. Combined capacity is 1.22 mtpa against 45.4 mtpa of export, so the choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
@@ -3638,17 +3552,14 @@
       <c r="AM13" s="4" t="inlineStr"/>
       <c r="AN13" s="4" t="inlineStr"/>
       <c r="AO13" s="4" t="inlineStr"/>
-      <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="n">
         <v>25</v>
       </c>
-      <c r="AR13" t="inlineStr"/>
       <c r="AS13" s="4" t="inlineStr">
         <is>
           <t>NRCan records a 25 year export licence. No FortisBC or Tilbury entry appears in the CER application schedule - unresolved.</t>
         </is>
       </c>
-      <c r="AT13" t="inlineStr"/>
       <c r="AU13" t="inlineStr">
         <is>
           <t>T100000131044</t>
@@ -3732,7 +3643,6 @@
           <t>Tilbury Island</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Fortis Inc [100.0%]</t>
@@ -3751,7 +3661,6 @@
       <c r="N14" t="b">
         <v>0</v>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
         <v>2028</v>
       </c>
@@ -3796,27 +3705,21 @@
           <t>Port of Vancouver ship-to-ship bunkering</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr"/>
       <c r="AC14" s="4" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
       <c r="AE14" s="4" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>not_published</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ14" s="4" t="inlineStr">
         <is>
-          <t>Drive type not published. These are small peak-shaving, off-grid or bunkering facilities, several predating 2000. The model applies liquefaction_drive_default from Parameters. Combined capacity is 1.22 mtpa against 45.4 mtpa of export, so the choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
+          <t>previously classified as not_published. Drive type not published. These are small peak-shaving, off-grid or bunkering facilities, several predating 2000. The model applies liquefaction_drive_default from Parameters. Combined capacity is 1.22 mtpa against 45.4 mtpa of export, so the choice between gas turbine and electric moves the total by under 0.2 MtCO2e a year.</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
@@ -3832,15 +3735,11 @@
       <c r="AM14" s="4" t="inlineStr"/>
       <c r="AN14" s="4" t="inlineStr"/>
       <c r="AO14" s="4" t="inlineStr"/>
-      <c r="AP14" t="inlineStr"/>
-      <c r="AQ14" t="inlineStr"/>
-      <c r="AR14" t="inlineStr"/>
       <c r="AS14" s="4" t="inlineStr">
         <is>
           <t>Not listed by NRCan as an export project; no licence identified</t>
         </is>
       </c>
-      <c r="AT14" t="inlineStr"/>
       <c r="AU14" t="inlineStr">
         <is>
           <t>T100000131044</t>
@@ -3885,8 +3784,6 @@
           <t>Tilbury Marine Jetty</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" s="8" t="inlineStr">
         <is>
           <t>advanced_proposed</t>
@@ -3912,7 +3809,6 @@
           <t>Tilbury Island, Delta</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
@@ -3927,14 +3823,11 @@
       <c r="N15" t="b">
         <v>0</v>
       </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
       <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>NRCan records export licence as not applicable. WesPac Midstream-Vancouver LLC holds GL-310 (25 year, Delta BC, issued 2016), which likely relates to this project but the identity is not confirmed.</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" s="4" t="inlineStr">
         <is>
           <t>Not applicable - marine jetty infrastructure, no liquefaction capacity</t>
@@ -3946,24 +3839,15 @@
         </is>
       </c>
       <c r="U15" s="4" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
       <c r="W15" s="4" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
       <c r="Y15" s="4" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
       <c r="AC15" s="4" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
       <c r="AE15" s="4" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
           <t>export infrastructure (marine jetty)</t>
         </is>
       </c>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
       <c r="AJ15" s="4" t="inlineStr"/>
       <c r="AK15" t="inlineStr">
         <is>
@@ -3978,12 +3862,7 @@
       <c r="AM15" s="4" t="inlineStr"/>
       <c r="AN15" s="4" t="inlineStr"/>
       <c r="AO15" s="4" t="inlineStr"/>
-      <c r="AP15" t="inlineStr"/>
-      <c r="AQ15" t="inlineStr"/>
-      <c r="AR15" t="inlineStr"/>
       <c r="AS15" s="4" t="inlineStr"/>
-      <c r="AT15" t="inlineStr"/>
-      <c r="AU15" t="inlineStr"/>
       <c r="AV15" s="4" t="inlineStr"/>
       <c r="AW15" s="4" t="inlineStr">
         <is>
@@ -4023,8 +3902,6 @@
           <t>Marinvest Energy LNG Export Project (Baie-Comeau)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" s="9" t="inlineStr">
         <is>
           <t>early_proposed</t>
@@ -4073,8 +3950,6 @@
       <c r="N16" t="b">
         <v>0</v>
       </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" t="n">
         <v>10</v>
@@ -4111,10 +3986,7 @@
       <c r="Z16" t="n">
         <v>2980</v>
       </c>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
       <c r="AC16" s="4" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
       <c r="AE16" s="4" t="inlineStr">
         <is>
           <t>Route distance not sourced</t>
@@ -4135,12 +4007,12 @@
       </c>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>electric_planned</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ16" s="4" t="inlineStr">
         <is>
-          <t>Company reported to be planning its own wind farm. No filed plan.</t>
+          <t>previously classified as electric_planned. Company reported to be planning its own wind farm. No filed plan.</t>
         </is>
       </c>
       <c r="AK16" t="inlineStr">
@@ -4168,16 +4040,11 @@
           <t>Aspirational - no filed plan</t>
         </is>
       </c>
-      <c r="AP16" t="inlineStr"/>
-      <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr"/>
       <c r="AS16" s="4" t="inlineStr">
         <is>
           <t>No export licence. Has not applied.</t>
         </is>
       </c>
-      <c r="AT16" t="inlineStr"/>
-      <c r="AU16" t="inlineStr"/>
       <c r="AV16" s="4" t="inlineStr"/>
       <c r="AW16" s="4" t="inlineStr">
         <is>
@@ -4213,8 +4080,6 @@
           <t>Summit Lake PG LNG</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" s="9" t="inlineStr">
         <is>
           <t>early_proposed</t>
@@ -4263,8 +4128,6 @@
       <c r="N17" t="b">
         <v>0</v>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
       <c r="Q17" s="4" t="inlineStr">
         <is>
           <t>None - has not applied</t>
@@ -4305,10 +4168,7 @@
       <c r="Z17" t="n">
         <v>3800</v>
       </c>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
       <c r="AC17" s="4" t="inlineStr"/>
-      <c r="AD17" t="inlineStr"/>
       <c r="AE17" s="4" t="inlineStr">
         <is>
           <t>Rail leg has no analogue in the other projects and is not yet modelled</t>
@@ -4319,18 +4179,17 @@
           <t>export</t>
         </is>
       </c>
-      <c r="AG17" t="inlineStr"/>
       <c r="AH17" t="b">
         <v>1</v>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>electric_planned</t>
+          <t>gas_turbine</t>
         </is>
       </c>
       <c r="AJ17" s="4" t="inlineStr">
         <is>
-          <t>Project description references green electrical utilities. No agreement identified.</t>
+          <t>previously classified as electric_planned. Project description references green electrical utilities. No agreement identified.</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -4361,15 +4220,11 @@
       <c r="AP17" t="n">
         <v>30</v>
       </c>
-      <c r="AQ17" t="inlineStr"/>
-      <c r="AR17" t="inlineStr"/>
       <c r="AS17" s="4" t="inlineStr">
         <is>
           <t>No export licence. Has not applied. Proponent states a 30 year operating life in its impact assessment.</t>
         </is>
       </c>
-      <c r="AT17" t="inlineStr"/>
-      <c r="AU17" t="inlineStr"/>
       <c r="AV17" s="4" t="inlineStr"/>
       <c r="AW17" s="4" t="inlineStr">
         <is>
@@ -4413,8 +4268,6 @@
           <t>Fermeuse Energy FLNG Terminal</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" s="9" t="inlineStr">
         <is>
           <t>early_proposed</t>
@@ -4430,9 +4283,21 @@
           <t>Proposed floating LNG. MOU with Hanwha Ocean Jan 2026. No capacity disclosed. Approved marine base only, no LNG plant proposal filed.</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Newfoundland and Labrador</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Fermeuse Marine Base, Newfoundland and Labrador</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Fermeuse Energy Ltd</t>
+        </is>
+      </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Crown LNG Holdings Ltd; Fermeuse Energy Ltd</t>
@@ -4445,22 +4310,27 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
+      <c r="R18" t="n">
+        <v>5</v>
+      </c>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>Derived, not published. The proponent has not stated a liquefaction capacity. This figure is constrained by the gas resource: Fermeuse Energy states the project would develop 9.7 trillion cubic feet of offshore associated gas in the Jeanne d'Arc Basin, which is 275 billion cubic metres. At 1.38 bcm per mtpa, spread over the 40-year operating life assumed elsewhere in this register, that supports 5.0 mtpa. Two other approaches give higher figures and were not used: the same reserve over a 25-year life gives 8.0 mtpa, and benchmarking the stated US$12 to 15 billion capital cost against Ksi Lisims and Cedar gives 9 to 12 mtpa. An unsourced third-party table circulates a figure of 10 mtpa. The lowest defensible derivation is used.</t>
+        </is>
+      </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
           <t>overseas export</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
       <c r="X18" t="inlineStr">
         <is>
@@ -4475,42 +4345,46 @@
       <c r="Z18" t="n">
         <v>2470</v>
       </c>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
       <c r="AC18" s="4" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" s="4" t="inlineStr"/>
+      <c r="AE18" s="4" t="inlineStr">
+        <is>
+          <t>Floating LNG at the Fermeuse Marine Base, Newfoundland and Labrador. Crown LNG affiliate. Memorandum of understanding with Hanwha Ocean signed January 2026, targeting first production 2030 to 2031. The mayor of Fermeuse told CBC in February 2026 that the company had not contacted the town, and the chief executive has said the project still needs to secure its first private investment commitments.</t>
+        </is>
+      </c>
       <c r="AF18" t="inlineStr">
         <is>
+          <t>export, floating</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>gas_turbine</t>
+        </is>
+      </c>
+      <c r="AJ18" s="4" t="inlineStr">
+        <is>
+          <t>previously classified as not_published.</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" s="4" t="inlineStr"/>
-      <c r="AK18" t="inlineStr">
-        <is>
-          <t>export</t>
-        </is>
-      </c>
       <c r="AL18" s="4" t="inlineStr">
         <is>
-          <t>Assigned from end_use</t>
+          <t>Assigned from end_use. Recorded explicitly so chain selection is a decision in the register rather than a text match on free text.</t>
         </is>
       </c>
       <c r="AM18" s="4" t="inlineStr"/>
       <c r="AN18" s="4" t="inlineStr"/>
       <c r="AO18" s="4" t="inlineStr"/>
-      <c r="AP18" t="inlineStr"/>
-      <c r="AQ18" t="inlineStr"/>
-      <c r="AR18" t="inlineStr"/>
       <c r="AS18" s="4" t="inlineStr"/>
-      <c r="AT18" t="inlineStr"/>
       <c r="AU18" t="inlineStr">
         <is>
           <t>T100001061412</t>
@@ -4532,7 +4406,7 @@
       <c r="BA18" s="4" t="inlineStr"/>
       <c r="BB18" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Fermeuse_Energy_FLNG_Terminal | NGI, Eastern Canada LNG / Hanwha: https://naturalgasintel.com/news/eastern-canada-lng-back-in-focus-as-hanwha-enters-newfoundland-project/</t>
+          <t>Fermeuse Energy news release, 2 September 2025 | GEM Fermeuse Energy FLNG Terminal, https://www.gem.wiki/Fermeuse_Energy_FLNG_Terminal | CBC, 10 February 2026, https://www.cbc.ca/news/canada/newfoundland-labrador/fermeuse-lng-proposed-project-9.7082941 | GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | NGI, Eastern Canada LNG / Hanwha: https://naturalgasintel.com/news/eastern-canada-lng-back-in-focus-as-hanwha-enters-newfoundland-project/</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4456,6 @@
           <t>Saint John</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Repsol SA [100.0%]</t>
@@ -4598,8 +4471,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>2009</v>
       </c>
@@ -4618,7 +4489,6 @@
         </is>
       </c>
       <c r="U19" s="4" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
       <c r="W19" s="4" t="inlineStr"/>
       <c r="X19" t="inlineStr">
         <is>
@@ -4633,19 +4503,13 @@
       <c r="Z19" t="n">
         <v>3050</v>
       </c>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
       <c r="AC19" s="4" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
       <c r="AE19" s="4" t="inlineStr"/>
       <c r="AF19" t="inlineStr">
         <is>
           <t>import</t>
         </is>
       </c>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
       <c r="AJ19" s="4" t="inlineStr"/>
       <c r="AK19" t="inlineStr">
         <is>
@@ -4660,11 +4524,7 @@
       <c r="AM19" s="4" t="inlineStr"/>
       <c r="AN19" s="4" t="inlineStr"/>
       <c r="AO19" s="4" t="inlineStr"/>
-      <c r="AP19" t="inlineStr"/>
-      <c r="AQ19" t="inlineStr"/>
-      <c r="AR19" t="inlineStr"/>
       <c r="AS19" s="4" t="inlineStr"/>
-      <c r="AT19" t="inlineStr"/>
       <c r="AU19" t="inlineStr">
         <is>
           <t>T100000130349</t>
@@ -4736,7 +4596,6 @@
           <t>Prince Rupert</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Orca LNG Ltd [100.0%]</t>
@@ -4752,9 +4611,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" t="n">
         <v>30</v>
@@ -4770,15 +4626,9 @@
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
       <c r="Y20" s="4" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
-      <c r="AB20" t="inlineStr"/>
       <c r="AC20" s="4" t="inlineStr"/>
-      <c r="AD20" t="inlineStr"/>
       <c r="AE20" s="4" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
@@ -4790,19 +4640,12 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AH20" t="inlineStr"/>
-      <c r="AI20" t="inlineStr"/>
       <c r="AJ20" s="4" t="inlineStr"/>
-      <c r="AK20" t="inlineStr"/>
       <c r="AL20" s="4" t="inlineStr"/>
       <c r="AM20" s="4" t="inlineStr"/>
       <c r="AN20" s="4" t="inlineStr"/>
       <c r="AO20" s="4" t="inlineStr"/>
-      <c r="AP20" t="inlineStr"/>
-      <c r="AQ20" t="inlineStr"/>
-      <c r="AR20" t="inlineStr"/>
       <c r="AS20" s="4" t="inlineStr"/>
-      <c r="AT20" t="inlineStr"/>
       <c r="AU20" t="inlineStr">
         <is>
           <t>T100000130362</t>
@@ -4874,7 +4717,6 @@
           <t>Tuck Inlet, Prince Rupert</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Exxon Mobil Corp [50.0%]; Imperial Oil Ltd [50.0%]</t>
@@ -4890,9 +4732,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" s="4" t="inlineStr"/>
       <c r="R21" t="n">
         <v>30</v>
@@ -4908,35 +4747,21 @@
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
       <c r="W21" s="4" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
       <c r="Y21" s="4" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
-      <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr"/>
       <c r="AC21" s="4" t="inlineStr"/>
-      <c r="AD21" t="inlineStr"/>
       <c r="AE21" s="4" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG21" t="inlineStr"/>
-      <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
       <c r="AJ21" s="4" t="inlineStr"/>
-      <c r="AK21" t="inlineStr"/>
       <c r="AL21" s="4" t="inlineStr"/>
       <c r="AM21" s="4" t="inlineStr"/>
       <c r="AN21" s="4" t="inlineStr"/>
       <c r="AO21" s="4" t="inlineStr"/>
-      <c r="AP21" t="inlineStr"/>
-      <c r="AQ21" t="inlineStr"/>
-      <c r="AR21" t="inlineStr"/>
       <c r="AS21" s="4" t="inlineStr"/>
-      <c r="AT21" t="inlineStr"/>
       <c r="AU21" t="inlineStr">
         <is>
           <t>T100000130372</t>
@@ -5008,7 +4833,6 @@
           <t>Port Alberni</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" s="4" t="inlineStr">
         <is>
           <t>Steelhead LNG Corp [100.0%]</t>
@@ -5024,9 +4848,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
       <c r="Q22" s="4" t="inlineStr"/>
       <c r="R22" t="n">
         <v>24</v>
@@ -5042,35 +4863,21 @@
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
       <c r="W22" s="4" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
       <c r="Y22" s="4" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
       <c r="AC22" s="4" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
       <c r="AE22" s="4" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG22" t="inlineStr"/>
-      <c r="AH22" t="inlineStr"/>
-      <c r="AI22" t="inlineStr"/>
       <c r="AJ22" s="4" t="inlineStr"/>
-      <c r="AK22" t="inlineStr"/>
       <c r="AL22" s="4" t="inlineStr"/>
       <c r="AM22" s="4" t="inlineStr"/>
       <c r="AN22" s="4" t="inlineStr"/>
       <c r="AO22" s="4" t="inlineStr"/>
-      <c r="AP22" t="inlineStr"/>
-      <c r="AQ22" t="inlineStr"/>
-      <c r="AR22" t="inlineStr"/>
       <c r="AS22" s="4" t="inlineStr"/>
-      <c r="AT22" t="inlineStr"/>
       <c r="AU22" t="inlineStr">
         <is>
           <t>T100000130366</t>
@@ -5142,7 +4949,6 @@
           <t>Ridley Island, Prince Rupert</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Shell PLC [100.0%]</t>
@@ -5158,9 +4964,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
       <c r="Q23" s="4" t="inlineStr"/>
       <c r="R23" t="n">
         <v>21</v>
@@ -5176,35 +4979,21 @@
         </is>
       </c>
       <c r="U23" s="4" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
       <c r="W23" s="4" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
       <c r="Y23" s="4" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
       <c r="AC23" s="4" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
       <c r="AE23" s="4" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr"/>
-      <c r="AI23" t="inlineStr"/>
       <c r="AJ23" s="4" t="inlineStr"/>
-      <c r="AK23" t="inlineStr"/>
       <c r="AL23" s="4" t="inlineStr"/>
       <c r="AM23" s="4" t="inlineStr"/>
       <c r="AN23" s="4" t="inlineStr"/>
       <c r="AO23" s="4" t="inlineStr"/>
-      <c r="AP23" t="inlineStr"/>
-      <c r="AQ23" t="inlineStr"/>
-      <c r="AR23" t="inlineStr"/>
       <c r="AS23" s="4" t="inlineStr"/>
-      <c r="AT23" t="inlineStr"/>
       <c r="AU23" t="inlineStr">
         <is>
           <t>T100000130364</t>
@@ -5253,17 +5042,17 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>inactive</t>
+          <t>early_proposed</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inactive</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Cancelled 2019 per GEM.</t>
+          <t>Early-stage proposal. Moved from inactive to early_proposed pending verification. No current filing or proponent activity was located in a review of news and regulatory sources in August 2026, and this classification should be revisited.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -5273,10 +5062,14 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Campbell River</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
+          <t>Campbell River, British Columbia</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Rockyview Resources Inc.</t>
+        </is>
+      </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
           <t>BV Investment Partners LP</t>
@@ -5284,18 +5077,16 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="n">
-        <v>2030</v>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
       </c>
       <c r="Q24" s="4" t="inlineStr"/>
       <c r="R24" t="n">
@@ -5303,7 +5094,7 @@
       </c>
       <c r="S24" s="4" t="inlineStr">
         <is>
-          <t>nameplate (GEM)</t>
+          <t>20 mtpa as recorded in Global Energy Monitor's Global Gas Infrastructure Tracker.</t>
         </is>
       </c>
       <c r="T24" s="4" t="inlineStr">
@@ -5312,35 +5103,43 @@
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
       <c r="W24" s="4" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
       <c r="Y24" s="4" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
       <c r="AC24" s="4" t="inlineStr"/>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" s="4" t="inlineStr"/>
+      <c r="AE24" s="4" t="inlineStr">
+        <is>
+          <t>Least verified asset in the register. GEM records 20 mtpa at Campbell River; no current filing or proponent activity was located in August 2026.</t>
+        </is>
+      </c>
       <c r="AF24" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG24" t="inlineStr"/>
-      <c r="AH24" t="inlineStr"/>
-      <c r="AI24" t="inlineStr"/>
-      <c r="AJ24" s="4" t="inlineStr"/>
-      <c r="AK24" t="inlineStr"/>
-      <c r="AL24" s="4" t="inlineStr"/>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>gas_turbine</t>
+        </is>
+      </c>
+      <c r="AJ24" s="4" t="inlineStr">
+        <is>
+          <t>previously classified as not_published.</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>export</t>
+        </is>
+      </c>
+      <c r="AL24" s="4" t="inlineStr">
+        <is>
+          <t>Assigned from end_use. Recorded explicitly so chain selection is a decision in the register rather than a text match on free text.</t>
+        </is>
+      </c>
       <c r="AM24" s="4" t="inlineStr"/>
       <c r="AN24" s="4" t="inlineStr"/>
       <c r="AO24" s="4" t="inlineStr"/>
-      <c r="AP24" t="inlineStr"/>
-      <c r="AQ24" t="inlineStr"/>
-      <c r="AR24" t="inlineStr"/>
       <c r="AS24" s="4" t="inlineStr"/>
-      <c r="AT24" t="inlineStr"/>
       <c r="AU24" t="inlineStr">
         <is>
           <t>T100000130351</t>
@@ -5412,7 +5211,6 @@
           <t>Kitsault</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Kitsault Energy Ltd [100.0%]</t>
@@ -5428,9 +5226,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
       <c r="Q25" s="4" t="inlineStr"/>
       <c r="R25" t="n">
         <v>20</v>
@@ -5446,35 +5241,21 @@
         </is>
       </c>
       <c r="U25" s="4" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
       <c r="W25" s="4" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
       <c r="Y25" s="4" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
       <c r="AC25" s="4" t="inlineStr"/>
-      <c r="AD25" t="inlineStr"/>
       <c r="AE25" s="4" t="inlineStr"/>
       <c r="AF25" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG25" t="inlineStr"/>
-      <c r="AH25" t="inlineStr"/>
-      <c r="AI25" t="inlineStr"/>
       <c r="AJ25" s="4" t="inlineStr"/>
-      <c r="AK25" t="inlineStr"/>
       <c r="AL25" s="4" t="inlineStr"/>
       <c r="AM25" s="4" t="inlineStr"/>
       <c r="AN25" s="4" t="inlineStr"/>
       <c r="AO25" s="4" t="inlineStr"/>
-      <c r="AP25" t="inlineStr"/>
-      <c r="AQ25" t="inlineStr"/>
-      <c r="AR25" t="inlineStr"/>
       <c r="AS25" s="4" t="inlineStr"/>
-      <c r="AT25" t="inlineStr"/>
       <c r="AU25" t="inlineStr">
         <is>
           <t>T100000130357</t>
@@ -5536,7 +5317,6 @@
           <t>Cancelled 2021 per GEM.</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
@@ -5566,7 +5346,6 @@
           <t>2023</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
       <c r="Q26" s="4" t="inlineStr"/>
       <c r="R26" t="n">
         <v>18</v>
@@ -5582,35 +5361,21 @@
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
       <c r="W26" s="4" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
       <c r="Y26" s="4" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="inlineStr"/>
-      <c r="AB26" t="inlineStr"/>
       <c r="AC26" s="4" t="inlineStr"/>
-      <c r="AD26" t="inlineStr"/>
       <c r="AE26" s="4" t="inlineStr"/>
       <c r="AF26" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG26" t="inlineStr"/>
-      <c r="AH26" t="inlineStr"/>
-      <c r="AI26" t="inlineStr"/>
       <c r="AJ26" s="4" t="inlineStr"/>
-      <c r="AK26" t="inlineStr"/>
       <c r="AL26" s="4" t="inlineStr"/>
       <c r="AM26" s="4" t="inlineStr"/>
       <c r="AN26" s="4" t="inlineStr"/>
       <c r="AO26" s="4" t="inlineStr"/>
-      <c r="AP26" t="inlineStr"/>
-      <c r="AQ26" t="inlineStr"/>
-      <c r="AR26" t="inlineStr"/>
       <c r="AS26" s="4" t="inlineStr"/>
-      <c r="AT26" t="inlineStr"/>
       <c r="AU26" t="inlineStr">
         <is>
           <t>T100000130356</t>
@@ -5682,7 +5447,6 @@
           <t>Lelu Island</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Petroliam Nasional Bhd</t>
@@ -5698,9 +5462,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
       <c r="Q27" s="4" t="inlineStr"/>
       <c r="R27" t="n">
         <v>18</v>
@@ -5716,35 +5477,21 @@
         </is>
       </c>
       <c r="U27" s="4" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
       <c r="W27" s="4" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
       <c r="Y27" s="4" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
-      <c r="AB27" t="inlineStr"/>
       <c r="AC27" s="4" t="inlineStr"/>
-      <c r="AD27" t="inlineStr"/>
       <c r="AE27" s="4" t="inlineStr"/>
       <c r="AF27" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG27" t="inlineStr"/>
-      <c r="AH27" t="inlineStr"/>
-      <c r="AI27" t="inlineStr"/>
       <c r="AJ27" s="4" t="inlineStr"/>
-      <c r="AK27" t="inlineStr"/>
       <c r="AL27" s="4" t="inlineStr"/>
       <c r="AM27" s="4" t="inlineStr"/>
       <c r="AN27" s="4" t="inlineStr"/>
       <c r="AO27" s="4" t="inlineStr"/>
-      <c r="AP27" t="inlineStr"/>
-      <c r="AQ27" t="inlineStr"/>
-      <c r="AR27" t="inlineStr"/>
       <c r="AS27" s="4" t="inlineStr"/>
-      <c r="AT27" t="inlineStr"/>
       <c r="AU27" t="inlineStr">
         <is>
           <t>T100000130363</t>
@@ -5781,8 +5528,6 @@
           <t>Atlantic Coast LNG Terminal</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -5808,7 +5553,6 @@
           <t>Byers Cove</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" s="4" t="inlineStr">
         <is>
           <t>A.C. LNG Inc [100.0%]</t>
@@ -5824,8 +5568,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
         <v>2024</v>
       </c>
@@ -5844,15 +5586,9 @@
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
       <c r="W28" s="4" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
       <c r="Y28" s="4" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
-      <c r="AB28" t="inlineStr"/>
       <c r="AC28" s="4" t="inlineStr"/>
-      <c r="AD28" t="inlineStr"/>
       <c r="AE28" s="4" t="inlineStr"/>
       <c r="AF28" t="inlineStr">
         <is>
@@ -5864,19 +5600,12 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AH28" t="inlineStr"/>
-      <c r="AI28" t="inlineStr"/>
       <c r="AJ28" s="4" t="inlineStr"/>
-      <c r="AK28" t="inlineStr"/>
       <c r="AL28" s="4" t="inlineStr"/>
       <c r="AM28" s="4" t="inlineStr"/>
       <c r="AN28" s="4" t="inlineStr"/>
       <c r="AO28" s="4" t="inlineStr"/>
-      <c r="AP28" t="inlineStr"/>
-      <c r="AQ28" t="inlineStr"/>
-      <c r="AR28" t="inlineStr"/>
       <c r="AS28" s="4" t="inlineStr"/>
-      <c r="AT28" t="inlineStr"/>
       <c r="AU28" t="inlineStr">
         <is>
           <t>T100000130345</t>
@@ -5935,7 +5664,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Cancelled 2018 per GEM.</t>
+          <t>Confirmed cancelled. Woodside declined to renew its sole proponent agreement, which expired 15 January 2018. The Impact Assessment Agency of Canada formally terminated the federal environmental assessment on 5 April 2018 at the proponent's own request.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -5948,7 +5677,6 @@
           <t>Grassy Point</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
       <c r="K29" s="4" t="inlineStr">
         <is>
           <t>Woodside Energy Group Ltd [100.0%]</t>
@@ -5961,12 +5689,9 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
+          <t>2026-08</t>
+        </is>
+      </c>
       <c r="Q29" s="4" t="inlineStr"/>
       <c r="R29" t="n">
         <v>15</v>
@@ -5982,35 +5707,21 @@
         </is>
       </c>
       <c r="U29" s="4" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
       <c r="W29" s="4" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
       <c r="Y29" s="4" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
-      <c r="AB29" t="inlineStr"/>
       <c r="AC29" s="4" t="inlineStr"/>
-      <c r="AD29" t="inlineStr"/>
       <c r="AE29" s="4" t="inlineStr"/>
       <c r="AF29" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG29" t="inlineStr"/>
-      <c r="AH29" t="inlineStr"/>
-      <c r="AI29" t="inlineStr"/>
       <c r="AJ29" s="4" t="inlineStr"/>
-      <c r="AK29" t="inlineStr"/>
       <c r="AL29" s="4" t="inlineStr"/>
       <c r="AM29" s="4" t="inlineStr"/>
       <c r="AN29" s="4" t="inlineStr"/>
       <c r="AO29" s="4" t="inlineStr"/>
-      <c r="AP29" t="inlineStr"/>
-      <c r="AQ29" t="inlineStr"/>
-      <c r="AR29" t="inlineStr"/>
       <c r="AS29" s="4" t="inlineStr"/>
-      <c r="AT29" t="inlineStr"/>
       <c r="AU29" t="inlineStr">
         <is>
           <t>T100000130355</t>
@@ -6032,7 +5743,7 @@
       <c r="BA29" s="4" t="inlineStr"/>
       <c r="BB29" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Grassy_Point_LNG_Terminal</t>
+          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Grassy_Point_LNG_Terminal | IAAC registry, https://iaac-aeic.gc.ca/050/evaluations/proj/80089</t>
         </is>
       </c>
     </row>
@@ -6082,7 +5793,6 @@
           <t>Delusion Bay</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" s="4" t="inlineStr">
         <is>
           <t>China National Offshore Oil  Corp [60.0%]; INPEX Corp [20.0%]; JGC Holdings Corp [20.0%]</t>
@@ -6098,9 +5808,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
       <c r="Q30" s="4" t="inlineStr"/>
       <c r="R30" t="n">
         <v>12</v>
@@ -6116,35 +5823,21 @@
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
       <c r="W30" s="4" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
       <c r="Y30" s="4" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="inlineStr"/>
-      <c r="AB30" t="inlineStr"/>
       <c r="AC30" s="4" t="inlineStr"/>
-      <c r="AD30" t="inlineStr"/>
       <c r="AE30" s="4" t="inlineStr"/>
       <c r="AF30" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG30" t="inlineStr"/>
-      <c r="AH30" t="inlineStr"/>
-      <c r="AI30" t="inlineStr"/>
       <c r="AJ30" s="4" t="inlineStr"/>
-      <c r="AK30" t="inlineStr"/>
       <c r="AL30" s="4" t="inlineStr"/>
       <c r="AM30" s="4" t="inlineStr"/>
       <c r="AN30" s="4" t="inlineStr"/>
       <c r="AO30" s="4" t="inlineStr"/>
-      <c r="AP30" t="inlineStr"/>
-      <c r="AQ30" t="inlineStr"/>
-      <c r="AR30" t="inlineStr"/>
       <c r="AS30" s="4" t="inlineStr"/>
-      <c r="AT30" t="inlineStr"/>
       <c r="AU30" t="inlineStr">
         <is>
           <t>T100000130346</t>
@@ -6216,7 +5909,6 @@
           <t>Delusion Bay</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" s="4" t="inlineStr">
         <is>
           <t>China National Offshore Oil  Corp [60.0%]; INPEX Corp [20.0%]; JGC Holdings Corp [20.0%]</t>
@@ -6232,9 +5924,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
       <c r="Q31" s="4" t="inlineStr"/>
       <c r="R31" t="n">
         <v>12</v>
@@ -6250,35 +5939,21 @@
         </is>
       </c>
       <c r="U31" s="4" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
       <c r="W31" s="4" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
       <c r="Y31" s="4" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr"/>
-      <c r="AB31" t="inlineStr"/>
       <c r="AC31" s="4" t="inlineStr"/>
-      <c r="AD31" t="inlineStr"/>
       <c r="AE31" s="4" t="inlineStr"/>
       <c r="AF31" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG31" t="inlineStr"/>
-      <c r="AH31" t="inlineStr"/>
-      <c r="AI31" t="inlineStr"/>
       <c r="AJ31" s="4" t="inlineStr"/>
-      <c r="AK31" t="inlineStr"/>
       <c r="AL31" s="4" t="inlineStr"/>
       <c r="AM31" s="4" t="inlineStr"/>
       <c r="AN31" s="4" t="inlineStr"/>
       <c r="AO31" s="4" t="inlineStr"/>
-      <c r="AP31" t="inlineStr"/>
-      <c r="AQ31" t="inlineStr"/>
-      <c r="AR31" t="inlineStr"/>
       <c r="AS31" s="4" t="inlineStr"/>
-      <c r="AT31" t="inlineStr"/>
       <c r="AU31" t="inlineStr">
         <is>
           <t>T100000130346</t>
@@ -6337,7 +6012,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Cancelled 2023 per GEM.</t>
+          <t>Confirmed cancelled as LNG. Acquired by Buckeye Partners in July 2022 and converted to a green hydrogen and ammonia facility. Nova Scotia granted environmental assessment approval for the hydrogen project in April 2023. The proponent's own site states the LNG tank foundations will be repurposed as ammonia storage.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -6350,7 +6025,6 @@
           <t>Point Tupper</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
       <c r="K32" s="4" t="inlineStr">
         <is>
           <t>IFM Global Infrastructure Fund</t>
@@ -6363,12 +6037,9 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
+          <t>2026-08</t>
+        </is>
+      </c>
       <c r="Q32" s="4" t="inlineStr"/>
       <c r="R32" t="n">
         <v>12</v>
@@ -6384,35 +6055,21 @@
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
       <c r="W32" s="4" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
       <c r="Y32" s="4" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="inlineStr"/>
-      <c r="AB32" t="inlineStr"/>
       <c r="AC32" s="4" t="inlineStr"/>
-      <c r="AD32" t="inlineStr"/>
       <c r="AE32" s="4" t="inlineStr"/>
       <c r="AF32" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG32" t="inlineStr"/>
-      <c r="AH32" t="inlineStr"/>
-      <c r="AI32" t="inlineStr"/>
       <c r="AJ32" s="4" t="inlineStr"/>
-      <c r="AK32" t="inlineStr"/>
       <c r="AL32" s="4" t="inlineStr"/>
       <c r="AM32" s="4" t="inlineStr"/>
       <c r="AN32" s="4" t="inlineStr"/>
       <c r="AO32" s="4" t="inlineStr"/>
-      <c r="AP32" t="inlineStr"/>
-      <c r="AQ32" t="inlineStr"/>
-      <c r="AR32" t="inlineStr"/>
       <c r="AS32" s="4" t="inlineStr"/>
-      <c r="AT32" t="inlineStr"/>
       <c r="AU32" t="inlineStr">
         <is>
           <t>T100000130347</t>
@@ -6434,7 +6091,7 @@
       <c r="BA32" s="4" t="inlineStr"/>
       <c r="BB32" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Bear_Head_LNG_Terminal</t>
+          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Bear_Head_LNG_Terminal | Nova Scotia EA registry, https://novascotia.ca/nse/ea/bear-head-energy/ | Bear Head Energy, https://www.bearheadenergy.ca/our-project</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6141,6 @@
           <t>Port Saguenay</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Breyer Capital LLC [50.0%]; Freestone International LLC [50.0%]</t>
@@ -6500,9 +6156,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
       <c r="Q33" s="4" t="inlineStr"/>
       <c r="R33" t="n">
         <v>11</v>
@@ -6518,35 +6171,21 @@
         </is>
       </c>
       <c r="U33" s="4" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
       <c r="W33" s="4" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
       <c r="Y33" s="4" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="inlineStr"/>
-      <c r="AB33" t="inlineStr"/>
       <c r="AC33" s="4" t="inlineStr"/>
-      <c r="AD33" t="inlineStr"/>
       <c r="AE33" s="4" t="inlineStr"/>
       <c r="AF33" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG33" t="inlineStr"/>
-      <c r="AH33" t="inlineStr"/>
-      <c r="AI33" t="inlineStr"/>
       <c r="AJ33" s="4" t="inlineStr"/>
-      <c r="AK33" t="inlineStr"/>
       <c r="AL33" s="4" t="inlineStr"/>
       <c r="AM33" s="4" t="inlineStr"/>
       <c r="AN33" s="4" t="inlineStr"/>
       <c r="AO33" s="4" t="inlineStr"/>
-      <c r="AP33" t="inlineStr"/>
-      <c r="AQ33" t="inlineStr"/>
-      <c r="AR33" t="inlineStr"/>
       <c r="AS33" s="4" t="inlineStr"/>
-      <c r="AT33" t="inlineStr"/>
       <c r="AU33" t="inlineStr">
         <is>
           <t>T100000130630</t>
@@ -6618,7 +6257,6 @@
           <t>Saint John</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Repsol SA [100.0%]</t>
@@ -6634,9 +6272,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
       <c r="Q34" s="4" t="inlineStr"/>
       <c r="R34" t="n">
         <v>7.5</v>
@@ -6652,7 +6287,6 @@
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
-      <c r="V34" t="inlineStr"/>
       <c r="W34" s="4" t="inlineStr"/>
       <c r="X34" t="inlineStr">
         <is>
@@ -6667,30 +6301,19 @@
       <c r="Z34" t="n">
         <v>3050</v>
       </c>
-      <c r="AA34" t="inlineStr"/>
-      <c r="AB34" t="inlineStr"/>
       <c r="AC34" s="4" t="inlineStr"/>
-      <c r="AD34" t="inlineStr"/>
       <c r="AE34" s="4" t="inlineStr"/>
       <c r="AF34" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG34" t="inlineStr"/>
-      <c r="AH34" t="inlineStr"/>
-      <c r="AI34" t="inlineStr"/>
       <c r="AJ34" s="4" t="inlineStr"/>
-      <c r="AK34" t="inlineStr"/>
       <c r="AL34" s="4" t="inlineStr"/>
       <c r="AM34" s="4" t="inlineStr"/>
       <c r="AN34" s="4" t="inlineStr"/>
       <c r="AO34" s="4" t="inlineStr"/>
-      <c r="AP34" t="inlineStr"/>
-      <c r="AQ34" t="inlineStr"/>
-      <c r="AR34" t="inlineStr"/>
       <c r="AS34" s="4" t="inlineStr"/>
-      <c r="AT34" t="inlineStr"/>
       <c r="AU34" t="inlineStr">
         <is>
           <t>T100000130349</t>
@@ -6727,8 +6350,6 @@
           <t>Malahat LNG Terminal</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -6754,7 +6375,6 @@
           <t>Victoria</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" s="4" t="inlineStr">
         <is>
           <t>Steelhead LNG Corp [100.0%]</t>
@@ -6770,9 +6390,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
       <c r="Q35" s="4" t="inlineStr"/>
       <c r="R35" t="n">
         <v>6</v>
@@ -6788,35 +6405,21 @@
         </is>
       </c>
       <c r="U35" s="4" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
       <c r="W35" s="4" t="inlineStr"/>
-      <c r="X35" t="inlineStr"/>
       <c r="Y35" s="4" t="inlineStr"/>
-      <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="inlineStr"/>
-      <c r="AB35" t="inlineStr"/>
       <c r="AC35" s="4" t="inlineStr"/>
-      <c r="AD35" t="inlineStr"/>
       <c r="AE35" s="4" t="inlineStr"/>
       <c r="AF35" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG35" t="inlineStr"/>
-      <c r="AH35" t="inlineStr"/>
-      <c r="AI35" t="inlineStr"/>
       <c r="AJ35" s="4" t="inlineStr"/>
-      <c r="AK35" t="inlineStr"/>
       <c r="AL35" s="4" t="inlineStr"/>
       <c r="AM35" s="4" t="inlineStr"/>
       <c r="AN35" s="4" t="inlineStr"/>
       <c r="AO35" s="4" t="inlineStr"/>
-      <c r="AP35" t="inlineStr"/>
-      <c r="AQ35" t="inlineStr"/>
-      <c r="AR35" t="inlineStr"/>
       <c r="AS35" s="4" t="inlineStr"/>
-      <c r="AT35" t="inlineStr"/>
       <c r="AU35" t="inlineStr">
         <is>
           <t>T100000130359</t>
@@ -6853,8 +6456,6 @@
           <t>Steelhead FSRU</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -6880,7 +6481,6 @@
           <t>Bamberton</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" s="4" t="inlineStr">
         <is>
           <t>Steelhead LNG Corp [100.0%]</t>
@@ -6896,9 +6496,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
       <c r="Q36" s="4" t="inlineStr"/>
       <c r="R36" t="n">
         <v>6</v>
@@ -6914,15 +6511,9 @@
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
       <c r="W36" s="4" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
       <c r="Y36" s="4" t="inlineStr"/>
-      <c r="Z36" t="inlineStr"/>
-      <c r="AA36" t="inlineStr"/>
-      <c r="AB36" t="inlineStr"/>
       <c r="AC36" s="4" t="inlineStr"/>
-      <c r="AD36" t="inlineStr"/>
       <c r="AE36" s="4" t="inlineStr"/>
       <c r="AF36" t="inlineStr">
         <is>
@@ -6934,19 +6525,12 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AH36" t="inlineStr"/>
-      <c r="AI36" t="inlineStr"/>
       <c r="AJ36" s="4" t="inlineStr"/>
-      <c r="AK36" t="inlineStr"/>
       <c r="AL36" s="4" t="inlineStr"/>
       <c r="AM36" s="4" t="inlineStr"/>
       <c r="AN36" s="4" t="inlineStr"/>
       <c r="AO36" s="4" t="inlineStr"/>
-      <c r="AP36" t="inlineStr"/>
-      <c r="AQ36" t="inlineStr"/>
-      <c r="AR36" t="inlineStr"/>
       <c r="AS36" s="4" t="inlineStr"/>
-      <c r="AT36" t="inlineStr"/>
       <c r="AU36" t="inlineStr">
         <is>
           <t>T100000130628</t>
@@ -7005,7 +6589,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Cancelled 2018 per GEM.</t>
+          <t>Confirmed cancelled. Woodside declined to renew its sole proponent agreement, which expired 15 January 2018. The Impact Assessment Agency of Canada formally terminated the federal environmental assessment on 5 April 2018 at the proponent's own request.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -7018,7 +6602,6 @@
           <t>Grassy Point</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" s="4" t="inlineStr">
         <is>
           <t>Woodside Energy Group Ltd [100.0%]</t>
@@ -7031,12 +6614,9 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
+          <t>2026-08</t>
+        </is>
+      </c>
       <c r="Q37" s="4" t="inlineStr"/>
       <c r="R37" t="n">
         <v>5</v>
@@ -7052,35 +6632,21 @@
         </is>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
       <c r="W37" s="4" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
       <c r="Y37" s="4" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
-      <c r="AA37" t="inlineStr"/>
-      <c r="AB37" t="inlineStr"/>
       <c r="AC37" s="4" t="inlineStr"/>
-      <c r="AD37" t="inlineStr"/>
       <c r="AE37" s="4" t="inlineStr"/>
       <c r="AF37" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG37" t="inlineStr"/>
-      <c r="AH37" t="inlineStr"/>
-      <c r="AI37" t="inlineStr"/>
       <c r="AJ37" s="4" t="inlineStr"/>
-      <c r="AK37" t="inlineStr"/>
       <c r="AL37" s="4" t="inlineStr"/>
       <c r="AM37" s="4" t="inlineStr"/>
       <c r="AN37" s="4" t="inlineStr"/>
       <c r="AO37" s="4" t="inlineStr"/>
-      <c r="AP37" t="inlineStr"/>
-      <c r="AQ37" t="inlineStr"/>
-      <c r="AR37" t="inlineStr"/>
       <c r="AS37" s="4" t="inlineStr"/>
-      <c r="AT37" t="inlineStr"/>
       <c r="AU37" t="inlineStr">
         <is>
           <t>T100000130355</t>
@@ -7102,7 +6668,7 @@
       <c r="BA37" s="4" t="inlineStr"/>
       <c r="BB37" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Grassy_Point_LNG_Terminal</t>
+          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Grassy_Point_LNG_Terminal | IAAC registry, https://iaac-aeic.gc.ca/050/evaluations/proj/80089</t>
         </is>
       </c>
     </row>
@@ -7152,7 +6718,6 @@
           <t>Stewart</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" s="4" t="inlineStr">
         <is>
           <t>Canada Stewart Energy Group Ltd [100.0%]</t>
@@ -7168,8 +6733,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="n">
         <v>2025</v>
       </c>
@@ -7188,15 +6751,9 @@
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
       <c r="W38" s="4" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
       <c r="Y38" s="4" t="inlineStr"/>
-      <c r="Z38" t="inlineStr"/>
-      <c r="AA38" t="inlineStr"/>
-      <c r="AB38" t="inlineStr"/>
       <c r="AC38" s="4" t="inlineStr"/>
-      <c r="AD38" t="inlineStr"/>
       <c r="AE38" s="4" t="inlineStr"/>
       <c r="AF38" t="inlineStr">
         <is>
@@ -7208,19 +6765,12 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AH38" t="inlineStr"/>
-      <c r="AI38" t="inlineStr"/>
       <c r="AJ38" s="4" t="inlineStr"/>
-      <c r="AK38" t="inlineStr"/>
       <c r="AL38" s="4" t="inlineStr"/>
       <c r="AM38" s="4" t="inlineStr"/>
       <c r="AN38" s="4" t="inlineStr"/>
       <c r="AO38" s="4" t="inlineStr"/>
-      <c r="AP38" t="inlineStr"/>
-      <c r="AQ38" t="inlineStr"/>
-      <c r="AR38" t="inlineStr"/>
       <c r="AS38" s="4" t="inlineStr"/>
-      <c r="AT38" t="inlineStr"/>
       <c r="AU38" t="inlineStr">
         <is>
           <t>T100000130367</t>
@@ -7292,7 +6842,6 @@
           <t>Stewart</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" s="4" t="inlineStr">
         <is>
           <t>Canada Stewart Energy Group Ltd [100.0%]</t>
@@ -7308,9 +6857,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
       <c r="Q39" s="4" t="inlineStr"/>
       <c r="R39" t="n">
         <v>5</v>
@@ -7326,15 +6872,9 @@
         </is>
       </c>
       <c r="U39" s="4" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
       <c r="W39" s="4" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
       <c r="Y39" s="4" t="inlineStr"/>
-      <c r="Z39" t="inlineStr"/>
-      <c r="AA39" t="inlineStr"/>
-      <c r="AB39" t="inlineStr"/>
       <c r="AC39" s="4" t="inlineStr"/>
-      <c r="AD39" t="inlineStr"/>
       <c r="AE39" s="4" t="inlineStr"/>
       <c r="AF39" t="inlineStr">
         <is>
@@ -7346,19 +6886,12 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AH39" t="inlineStr"/>
-      <c r="AI39" t="inlineStr"/>
       <c r="AJ39" s="4" t="inlineStr"/>
-      <c r="AK39" t="inlineStr"/>
       <c r="AL39" s="4" t="inlineStr"/>
       <c r="AM39" s="4" t="inlineStr"/>
       <c r="AN39" s="4" t="inlineStr"/>
       <c r="AO39" s="4" t="inlineStr"/>
-      <c r="AP39" t="inlineStr"/>
-      <c r="AQ39" t="inlineStr"/>
-      <c r="AR39" t="inlineStr"/>
       <c r="AS39" s="4" t="inlineStr"/>
-      <c r="AT39" t="inlineStr"/>
       <c r="AU39" t="inlineStr">
         <is>
           <t>T100000130367</t>
@@ -7430,7 +6963,6 @@
           <t>Prince Rupert</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" s="4" t="inlineStr">
         <is>
           <t>NewTimes Energy Ltd [100.0%]</t>
@@ -7446,9 +6978,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
       <c r="Q40" s="4" t="inlineStr"/>
       <c r="R40" t="n">
         <v>4</v>
@@ -7464,35 +6993,21 @@
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
       <c r="W40" s="4" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
       <c r="Y40" s="4" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
-      <c r="AA40" t="inlineStr"/>
-      <c r="AB40" t="inlineStr"/>
       <c r="AC40" s="4" t="inlineStr"/>
-      <c r="AD40" t="inlineStr"/>
       <c r="AE40" s="4" t="inlineStr"/>
       <c r="AF40" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG40" t="inlineStr"/>
-      <c r="AH40" t="inlineStr"/>
-      <c r="AI40" t="inlineStr"/>
       <c r="AJ40" s="4" t="inlineStr"/>
-      <c r="AK40" t="inlineStr"/>
       <c r="AL40" s="4" t="inlineStr"/>
       <c r="AM40" s="4" t="inlineStr"/>
       <c r="AN40" s="4" t="inlineStr"/>
       <c r="AO40" s="4" t="inlineStr"/>
-      <c r="AP40" t="inlineStr"/>
-      <c r="AQ40" t="inlineStr"/>
-      <c r="AR40" t="inlineStr"/>
       <c r="AS40" s="4" t="inlineStr"/>
-      <c r="AT40" t="inlineStr"/>
       <c r="AU40" t="inlineStr">
         <is>
           <t>T100000130360</t>
@@ -7564,7 +7079,6 @@
           <t>Prince Rupert</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" s="4" t="inlineStr">
         <is>
           <t>NewTimes Energy Ltd [100.0%]</t>
@@ -7580,9 +7094,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
       <c r="Q41" s="4" t="inlineStr"/>
       <c r="R41" t="n">
         <v>4</v>
@@ -7598,35 +7109,21 @@
         </is>
       </c>
       <c r="U41" s="4" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
       <c r="W41" s="4" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
       <c r="Y41" s="4" t="inlineStr"/>
-      <c r="Z41" t="inlineStr"/>
-      <c r="AA41" t="inlineStr"/>
-      <c r="AB41" t="inlineStr"/>
       <c r="AC41" s="4" t="inlineStr"/>
-      <c r="AD41" t="inlineStr"/>
       <c r="AE41" s="4" t="inlineStr"/>
       <c r="AF41" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG41" t="inlineStr"/>
-      <c r="AH41" t="inlineStr"/>
-      <c r="AI41" t="inlineStr"/>
       <c r="AJ41" s="4" t="inlineStr"/>
-      <c r="AK41" t="inlineStr"/>
       <c r="AL41" s="4" t="inlineStr"/>
       <c r="AM41" s="4" t="inlineStr"/>
       <c r="AN41" s="4" t="inlineStr"/>
       <c r="AO41" s="4" t="inlineStr"/>
-      <c r="AP41" t="inlineStr"/>
-      <c r="AQ41" t="inlineStr"/>
-      <c r="AR41" t="inlineStr"/>
       <c r="AS41" s="4" t="inlineStr"/>
-      <c r="AT41" t="inlineStr"/>
       <c r="AU41" t="inlineStr">
         <is>
           <t>T100000130360</t>
@@ -7698,7 +7195,6 @@
           <t>Prince Rupert</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" s="4" t="inlineStr">
         <is>
           <t>NewTimes Energy Ltd [100.0%]</t>
@@ -7714,9 +7210,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
       <c r="Q42" s="4" t="inlineStr"/>
       <c r="R42" t="n">
         <v>4</v>
@@ -7732,35 +7225,21 @@
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr"/>
-      <c r="V42" t="inlineStr"/>
       <c r="W42" s="4" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
       <c r="Y42" s="4" t="inlineStr"/>
-      <c r="Z42" t="inlineStr"/>
-      <c r="AA42" t="inlineStr"/>
-      <c r="AB42" t="inlineStr"/>
       <c r="AC42" s="4" t="inlineStr"/>
-      <c r="AD42" t="inlineStr"/>
       <c r="AE42" s="4" t="inlineStr"/>
       <c r="AF42" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG42" t="inlineStr"/>
-      <c r="AH42" t="inlineStr"/>
-      <c r="AI42" t="inlineStr"/>
       <c r="AJ42" s="4" t="inlineStr"/>
-      <c r="AK42" t="inlineStr"/>
       <c r="AL42" s="4" t="inlineStr"/>
       <c r="AM42" s="4" t="inlineStr"/>
       <c r="AN42" s="4" t="inlineStr"/>
       <c r="AO42" s="4" t="inlineStr"/>
-      <c r="AP42" t="inlineStr"/>
-      <c r="AQ42" t="inlineStr"/>
-      <c r="AR42" t="inlineStr"/>
       <c r="AS42" s="4" t="inlineStr"/>
-      <c r="AT42" t="inlineStr"/>
       <c r="AU42" t="inlineStr">
         <is>
           <t>T100000130360</t>
@@ -7797,8 +7276,6 @@
           <t>Placentia Bay FLNG Terminal</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -7824,7 +7301,6 @@
           <t>Arnold's Cove</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" s="4" t="inlineStr">
         <is>
           <t>LNG Newfoundland and Labrador Ltd</t>
@@ -7848,7 +7324,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr"/>
       <c r="Q43" s="4" t="inlineStr"/>
       <c r="R43" t="n">
         <v>4</v>
@@ -7864,15 +7339,9 @@
         </is>
       </c>
       <c r="U43" s="4" t="inlineStr"/>
-      <c r="V43" t="inlineStr"/>
       <c r="W43" s="4" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
       <c r="Y43" s="4" t="inlineStr"/>
-      <c r="Z43" t="inlineStr"/>
-      <c r="AA43" t="inlineStr"/>
-      <c r="AB43" t="inlineStr"/>
       <c r="AC43" s="4" t="inlineStr"/>
-      <c r="AD43" t="inlineStr"/>
       <c r="AE43" s="4" t="inlineStr"/>
       <c r="AF43" t="inlineStr">
         <is>
@@ -7884,19 +7353,12 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AH43" t="inlineStr"/>
-      <c r="AI43" t="inlineStr"/>
       <c r="AJ43" s="4" t="inlineStr"/>
-      <c r="AK43" t="inlineStr"/>
       <c r="AL43" s="4" t="inlineStr"/>
       <c r="AM43" s="4" t="inlineStr"/>
       <c r="AN43" s="4" t="inlineStr"/>
       <c r="AO43" s="4" t="inlineStr"/>
-      <c r="AP43" t="inlineStr"/>
-      <c r="AQ43" t="inlineStr"/>
-      <c r="AR43" t="inlineStr"/>
       <c r="AS43" s="4" t="inlineStr"/>
-      <c r="AT43" t="inlineStr"/>
       <c r="AU43" t="inlineStr">
         <is>
           <t>T100000131042</t>
@@ -7933,8 +7395,6 @@
           <t>Cacouna LNG Terminal</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -7960,7 +7420,6 @@
           <t>Gros Cacouna</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" s="4" t="inlineStr">
         <is>
           <t>Petro-Canada Inc; TC Energy Corp</t>
@@ -7976,9 +7435,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
       <c r="Q44" s="4" t="inlineStr"/>
       <c r="R44" t="n">
         <v>3.8</v>
@@ -7994,35 +7450,21 @@
         </is>
       </c>
       <c r="U44" s="4" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
       <c r="W44" s="4" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
       <c r="Y44" s="4" t="inlineStr"/>
-      <c r="Z44" t="inlineStr"/>
-      <c r="AA44" t="inlineStr"/>
-      <c r="AB44" t="inlineStr"/>
       <c r="AC44" s="4" t="inlineStr"/>
-      <c r="AD44" t="inlineStr"/>
       <c r="AE44" s="4" t="inlineStr"/>
       <c r="AF44" t="inlineStr">
         <is>
           <t>import</t>
         </is>
       </c>
-      <c r="AG44" t="inlineStr"/>
-      <c r="AH44" t="inlineStr"/>
-      <c r="AI44" t="inlineStr"/>
       <c r="AJ44" s="4" t="inlineStr"/>
-      <c r="AK44" t="inlineStr"/>
       <c r="AL44" s="4" t="inlineStr"/>
       <c r="AM44" s="4" t="inlineStr"/>
       <c r="AN44" s="4" t="inlineStr"/>
       <c r="AO44" s="4" t="inlineStr"/>
-      <c r="AP44" t="inlineStr"/>
-      <c r="AQ44" t="inlineStr"/>
-      <c r="AR44" t="inlineStr"/>
       <c r="AS44" s="4" t="inlineStr"/>
-      <c r="AT44" t="inlineStr"/>
       <c r="AU44" t="inlineStr">
         <is>
           <t>T100000130348</t>
@@ -8059,8 +7501,6 @@
           <t>Rabaska LNG Terminal</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -8086,7 +7526,6 @@
           <t>Lévis</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" s="4" t="inlineStr">
         <is>
           <t>Enbridge Inc; ENGIE SA; Gazprom PJSC; Énergir Inc</t>
@@ -8102,9 +7541,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
       <c r="Q45" s="4" t="inlineStr"/>
       <c r="R45" t="n">
         <v>3.8</v>
@@ -8120,35 +7556,21 @@
         </is>
       </c>
       <c r="U45" s="4" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
       <c r="W45" s="4" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
       <c r="Y45" s="4" t="inlineStr"/>
-      <c r="Z45" t="inlineStr"/>
-      <c r="AA45" t="inlineStr"/>
-      <c r="AB45" t="inlineStr"/>
       <c r="AC45" s="4" t="inlineStr"/>
-      <c r="AD45" t="inlineStr"/>
       <c r="AE45" s="4" t="inlineStr"/>
       <c r="AF45" t="inlineStr">
         <is>
           <t>import</t>
         </is>
       </c>
-      <c r="AG45" t="inlineStr"/>
-      <c r="AH45" t="inlineStr"/>
-      <c r="AI45" t="inlineStr"/>
       <c r="AJ45" s="4" t="inlineStr"/>
-      <c r="AK45" t="inlineStr"/>
       <c r="AL45" s="4" t="inlineStr"/>
       <c r="AM45" s="4" t="inlineStr"/>
       <c r="AN45" s="4" t="inlineStr"/>
       <c r="AO45" s="4" t="inlineStr"/>
-      <c r="AP45" t="inlineStr"/>
-      <c r="AQ45" t="inlineStr"/>
-      <c r="AR45" t="inlineStr"/>
       <c r="AS45" s="4" t="inlineStr"/>
-      <c r="AT45" t="inlineStr"/>
       <c r="AU45" t="inlineStr">
         <is>
           <t>T100000130365</t>
@@ -8185,8 +7607,6 @@
           <t>Texada LNG Terminal</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -8212,7 +7632,6 @@
           <t>Texada Island</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" s="4" t="inlineStr">
         <is>
           <t>WestPac LNG Corp [100.0%]</t>
@@ -8228,9 +7647,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
       <c r="Q46" s="4" t="inlineStr"/>
       <c r="R46" t="n">
         <v>3.8</v>
@@ -8246,35 +7662,21 @@
         </is>
       </c>
       <c r="U46" s="4" t="inlineStr"/>
-      <c r="V46" t="inlineStr"/>
       <c r="W46" s="4" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
       <c r="Y46" s="4" t="inlineStr"/>
-      <c r="Z46" t="inlineStr"/>
-      <c r="AA46" t="inlineStr"/>
-      <c r="AB46" t="inlineStr"/>
       <c r="AC46" s="4" t="inlineStr"/>
-      <c r="AD46" t="inlineStr"/>
       <c r="AE46" s="4" t="inlineStr"/>
       <c r="AF46" t="inlineStr">
         <is>
           <t>import</t>
         </is>
       </c>
-      <c r="AG46" t="inlineStr"/>
-      <c r="AH46" t="inlineStr"/>
-      <c r="AI46" t="inlineStr"/>
       <c r="AJ46" s="4" t="inlineStr"/>
-      <c r="AK46" t="inlineStr"/>
       <c r="AL46" s="4" t="inlineStr"/>
       <c r="AM46" s="4" t="inlineStr"/>
       <c r="AN46" s="4" t="inlineStr"/>
       <c r="AO46" s="4" t="inlineStr"/>
-      <c r="AP46" t="inlineStr"/>
-      <c r="AQ46" t="inlineStr"/>
-      <c r="AR46" t="inlineStr"/>
       <c r="AS46" s="4" t="inlineStr"/>
-      <c r="AT46" t="inlineStr"/>
       <c r="AU46" t="inlineStr">
         <is>
           <t>T100000130369</t>
@@ -8311,8 +7713,6 @@
           <t>Triton LNG Export Terminal</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -8338,7 +7738,6 @@
           <t>Douglas Channel</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
       <c r="K47" s="4" t="inlineStr">
         <is>
           <t>AltaGas Ltd [50.0%]; Idemitsu Kosan Co Ltd [50.0%]</t>
@@ -8357,8 +7756,6 @@
       <c r="N47" t="b">
         <v>0</v>
       </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
       <c r="Q47" s="4" t="inlineStr"/>
       <c r="R47" t="n">
         <v>2.3</v>
@@ -8374,35 +7771,21 @@
         </is>
       </c>
       <c r="U47" s="4" t="inlineStr"/>
-      <c r="V47" t="inlineStr"/>
       <c r="W47" s="4" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
       <c r="Y47" s="4" t="inlineStr"/>
-      <c r="Z47" t="inlineStr"/>
-      <c r="AA47" t="inlineStr"/>
-      <c r="AB47" t="inlineStr"/>
       <c r="AC47" s="4" t="inlineStr"/>
-      <c r="AD47" t="inlineStr"/>
       <c r="AE47" s="4" t="inlineStr"/>
       <c r="AF47" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG47" t="inlineStr"/>
-      <c r="AH47" t="inlineStr"/>
-      <c r="AI47" t="inlineStr"/>
       <c r="AJ47" s="4" t="inlineStr"/>
-      <c r="AK47" t="inlineStr"/>
       <c r="AL47" s="4" t="inlineStr"/>
       <c r="AM47" s="4" t="inlineStr"/>
       <c r="AN47" s="4" t="inlineStr"/>
       <c r="AO47" s="4" t="inlineStr"/>
-      <c r="AP47" t="inlineStr"/>
-      <c r="AQ47" t="inlineStr"/>
-      <c r="AR47" t="inlineStr"/>
       <c r="AS47" s="4" t="inlineStr"/>
-      <c r="AT47" t="inlineStr"/>
       <c r="AU47" t="inlineStr">
         <is>
           <t>T100000130370</t>
@@ -8439,8 +7822,6 @@
           <t>Watson Island LNG Terminal</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -8466,7 +7847,6 @@
           <t>Prince Rupert</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
       <c r="K48" s="4" t="inlineStr">
         <is>
           <t>Watson Island LNG Corp</t>
@@ -8482,9 +7862,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
       <c r="Q48" s="4" t="inlineStr"/>
       <c r="R48" t="n">
         <v>1</v>
@@ -8500,35 +7877,21 @@
         </is>
       </c>
       <c r="U48" s="4" t="inlineStr"/>
-      <c r="V48" t="inlineStr"/>
       <c r="W48" s="4" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
       <c r="Y48" s="4" t="inlineStr"/>
-      <c r="Z48" t="inlineStr"/>
-      <c r="AA48" t="inlineStr"/>
-      <c r="AB48" t="inlineStr"/>
       <c r="AC48" s="4" t="inlineStr"/>
-      <c r="AD48" t="inlineStr"/>
       <c r="AE48" s="4" t="inlineStr"/>
       <c r="AF48" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG48" t="inlineStr"/>
-      <c r="AH48" t="inlineStr"/>
-      <c r="AI48" t="inlineStr"/>
       <c r="AJ48" s="4" t="inlineStr"/>
-      <c r="AK48" t="inlineStr"/>
       <c r="AL48" s="4" t="inlineStr"/>
       <c r="AM48" s="4" t="inlineStr"/>
       <c r="AN48" s="4" t="inlineStr"/>
       <c r="AO48" s="4" t="inlineStr"/>
-      <c r="AP48" t="inlineStr"/>
-      <c r="AQ48" t="inlineStr"/>
-      <c r="AR48" t="inlineStr"/>
       <c r="AS48" s="4" t="inlineStr"/>
-      <c r="AT48" t="inlineStr"/>
       <c r="AU48" t="inlineStr">
         <is>
           <t>T100000130371</t>
@@ -8565,8 +7928,6 @@
           <t>Douglas Channel LNG Terminal</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -8592,7 +7953,6 @@
           <t>Douglas Channel</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
       <c r="K49" s="4" t="inlineStr">
         <is>
           <t>AltaGas Ltd; Electricité de France SA; Exmar NV; Idemitsu Kosan Co Ltd</t>
@@ -8608,9 +7968,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
       <c r="Q49" s="4" t="inlineStr"/>
       <c r="R49" t="n">
         <v>0.55</v>
@@ -8626,35 +7983,21 @@
         </is>
       </c>
       <c r="U49" s="4" t="inlineStr"/>
-      <c r="V49" t="inlineStr"/>
       <c r="W49" s="4" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
       <c r="Y49" s="4" t="inlineStr"/>
-      <c r="Z49" t="inlineStr"/>
-      <c r="AA49" t="inlineStr"/>
-      <c r="AB49" t="inlineStr"/>
       <c r="AC49" s="4" t="inlineStr"/>
-      <c r="AD49" t="inlineStr"/>
       <c r="AE49" s="4" t="inlineStr"/>
       <c r="AF49" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG49" t="inlineStr"/>
-      <c r="AH49" t="inlineStr"/>
-      <c r="AI49" t="inlineStr"/>
       <c r="AJ49" s="4" t="inlineStr"/>
-      <c r="AK49" t="inlineStr"/>
       <c r="AL49" s="4" t="inlineStr"/>
       <c r="AM49" s="4" t="inlineStr"/>
       <c r="AN49" s="4" t="inlineStr"/>
       <c r="AO49" s="4" t="inlineStr"/>
-      <c r="AP49" t="inlineStr"/>
-      <c r="AQ49" t="inlineStr"/>
-      <c r="AR49" t="inlineStr"/>
       <c r="AS49" s="4" t="inlineStr"/>
-      <c r="AT49" t="inlineStr"/>
       <c r="AU49" t="inlineStr">
         <is>
           <t>T100000130352</t>
@@ -8726,7 +8069,6 @@
           <t>Bécancour</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
       <c r="K50" s="4" t="inlineStr">
         <is>
           <t>Stolt LNGaz [100.0%]</t>
@@ -8742,9 +8084,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
       <c r="Q50" s="4" t="inlineStr"/>
       <c r="R50" t="n">
         <v>0.5</v>
@@ -8760,35 +8099,21 @@
         </is>
       </c>
       <c r="U50" s="4" t="inlineStr"/>
-      <c r="V50" t="inlineStr"/>
       <c r="W50" s="4" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
       <c r="Y50" s="4" t="inlineStr"/>
-      <c r="Z50" t="inlineStr"/>
-      <c r="AA50" t="inlineStr"/>
-      <c r="AB50" t="inlineStr"/>
       <c r="AC50" s="4" t="inlineStr"/>
-      <c r="AD50" t="inlineStr"/>
       <c r="AE50" s="4" t="inlineStr"/>
       <c r="AF50" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG50" t="inlineStr"/>
-      <c r="AH50" t="inlineStr"/>
-      <c r="AI50" t="inlineStr"/>
       <c r="AJ50" s="4" t="inlineStr"/>
-      <c r="AK50" t="inlineStr"/>
       <c r="AL50" s="4" t="inlineStr"/>
       <c r="AM50" s="4" t="inlineStr"/>
       <c r="AN50" s="4" t="inlineStr"/>
       <c r="AO50" s="4" t="inlineStr"/>
-      <c r="AP50" t="inlineStr"/>
-      <c r="AQ50" t="inlineStr"/>
-      <c r="AR50" t="inlineStr"/>
       <c r="AS50" s="4" t="inlineStr"/>
-      <c r="AT50" t="inlineStr"/>
       <c r="AU50" t="inlineStr">
         <is>
           <t>T100000130368</t>
@@ -8825,8 +8150,6 @@
           <t>Port Edward LNG Terminal</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -8872,9 +8195,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
       <c r="Q51" s="4" t="inlineStr"/>
       <c r="R51" t="n">
         <v>0.3</v>
@@ -8890,35 +8210,21 @@
         </is>
       </c>
       <c r="U51" s="4" t="inlineStr"/>
-      <c r="V51" t="inlineStr"/>
       <c r="W51" s="4" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
       <c r="Y51" s="4" t="inlineStr"/>
-      <c r="Z51" t="inlineStr"/>
-      <c r="AA51" t="inlineStr"/>
-      <c r="AB51" t="inlineStr"/>
       <c r="AC51" s="4" t="inlineStr"/>
-      <c r="AD51" t="inlineStr"/>
       <c r="AE51" s="4" t="inlineStr"/>
       <c r="AF51" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG51" t="inlineStr"/>
-      <c r="AH51" t="inlineStr"/>
-      <c r="AI51" t="inlineStr"/>
       <c r="AJ51" s="4" t="inlineStr"/>
-      <c r="AK51" t="inlineStr"/>
       <c r="AL51" s="4" t="inlineStr"/>
       <c r="AM51" s="4" t="inlineStr"/>
       <c r="AN51" s="4" t="inlineStr"/>
       <c r="AO51" s="4" t="inlineStr"/>
-      <c r="AP51" t="inlineStr"/>
-      <c r="AQ51" t="inlineStr"/>
-      <c r="AR51" t="inlineStr"/>
       <c r="AS51" s="4" t="inlineStr"/>
-      <c r="AT51" t="inlineStr"/>
       <c r="AU51" t="inlineStr">
         <is>
           <t>T100000131127</t>
@@ -8955,8 +8261,6 @@
           <t>Skeena LNG Terminal</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -8982,7 +8286,6 @@
           <t>Skeena</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" s="4" t="inlineStr">
         <is>
           <t>unknown [55.0%]; China Sunshine Paper Holdings Co Ltd [45.0%]</t>
@@ -8998,9 +8301,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
       <c r="Q52" s="4" t="inlineStr"/>
       <c r="R52" t="n">
         <v>0.15</v>
@@ -9016,35 +8316,21 @@
         </is>
       </c>
       <c r="U52" s="4" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
       <c r="W52" s="4" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
       <c r="Y52" s="4" t="inlineStr"/>
-      <c r="Z52" t="inlineStr"/>
-      <c r="AA52" t="inlineStr"/>
-      <c r="AB52" t="inlineStr"/>
       <c r="AC52" s="4" t="inlineStr"/>
-      <c r="AD52" t="inlineStr"/>
       <c r="AE52" s="4" t="inlineStr"/>
       <c r="AF52" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG52" t="inlineStr"/>
-      <c r="AH52" t="inlineStr"/>
-      <c r="AI52" t="inlineStr"/>
       <c r="AJ52" s="4" t="inlineStr"/>
-      <c r="AK52" t="inlineStr"/>
       <c r="AL52" s="4" t="inlineStr"/>
       <c r="AM52" s="4" t="inlineStr"/>
       <c r="AN52" s="4" t="inlineStr"/>
       <c r="AO52" s="4" t="inlineStr"/>
-      <c r="AP52" t="inlineStr"/>
-      <c r="AQ52" t="inlineStr"/>
-      <c r="AR52" t="inlineStr"/>
       <c r="AS52" s="4" t="inlineStr"/>
-      <c r="AT52" t="inlineStr"/>
       <c r="AU52" t="inlineStr">
         <is>
           <t>T100000130939</t>
@@ -9103,7 +8389,7 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>Shelved. Pieridae Energy transferred the Nova Scotia assets and licensing; now held by Cavvy Energy Ltd.</t>
+          <t>Confirmed cancelled. Pieridae abandoned the project in 2023 after eleven years and sold the Goldboro subsidiary in July 2024 for CAD 12 million. The Uniper offtake agreement lapsed. GEM records as of June 2026 that the project has not been revived and is considered cancelled.</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -9116,7 +8402,6 @@
           <t>Goldboro</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" s="4" t="inlineStr">
         <is>
           <t>Cavvy Energy Ltd [100.0%]</t>
@@ -9124,12 +8409,12 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>shelved</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N53" t="b">
@@ -9140,9 +8425,7 @@
           <t>2021</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr"/>
       <c r="Q53" s="4" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
       <c r="S53" s="4" t="inlineStr"/>
       <c r="T53" s="4" t="inlineStr">
         <is>
@@ -9150,35 +8433,21 @@
         </is>
       </c>
       <c r="U53" s="4" t="inlineStr"/>
-      <c r="V53" t="inlineStr"/>
       <c r="W53" s="4" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
       <c r="Y53" s="4" t="inlineStr"/>
-      <c r="Z53" t="inlineStr"/>
-      <c r="AA53" t="inlineStr"/>
-      <c r="AB53" t="inlineStr"/>
       <c r="AC53" s="4" t="inlineStr"/>
-      <c r="AD53" t="inlineStr"/>
       <c r="AE53" s="4" t="inlineStr"/>
       <c r="AF53" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG53" t="inlineStr"/>
-      <c r="AH53" t="inlineStr"/>
-      <c r="AI53" t="inlineStr"/>
       <c r="AJ53" s="4" t="inlineStr"/>
-      <c r="AK53" t="inlineStr"/>
       <c r="AL53" s="4" t="inlineStr"/>
       <c r="AM53" s="4" t="inlineStr"/>
       <c r="AN53" s="4" t="inlineStr"/>
       <c r="AO53" s="4" t="inlineStr"/>
-      <c r="AP53" t="inlineStr"/>
-      <c r="AQ53" t="inlineStr"/>
-      <c r="AR53" t="inlineStr"/>
       <c r="AS53" s="4" t="inlineStr"/>
-      <c r="AT53" t="inlineStr"/>
       <c r="AU53" t="inlineStr">
         <is>
           <t>T100000130354</t>
@@ -9200,7 +8469,7 @@
       <c r="BA53" s="4" t="inlineStr"/>
       <c r="BB53" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Goldboro_LNG_Terminal</t>
+          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Goldboro_LNG_Terminal | CBC, https://www.cbc.ca/news/canada/nova-scotia/proposed-goldboro-lng-plant-abandoned-after-11-years-1.7038936 | GEM, https://www.gem.wiki/Goldboro_LNG_Terminal</t>
         </is>
       </c>
     </row>
@@ -9237,7 +8506,7 @@
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Shelved. Pieridae Energy transferred the Nova Scotia assets and licensing; now held by Cavvy Energy Ltd.</t>
+          <t>Confirmed cancelled. Pieridae abandoned the project in 2023 after eleven years and sold the Goldboro subsidiary in July 2024 for CAD 12 million. The Uniper offtake agreement lapsed. GEM records as of June 2026 that the project has not been revived and is considered cancelled.</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -9250,7 +8519,6 @@
           <t>Goldboro</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" s="4" t="inlineStr">
         <is>
           <t>Cavvy Energy Ltd [100.0%]</t>
@@ -9258,12 +8526,12 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>shelved</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N54" t="b">
@@ -9274,9 +8542,7 @@
           <t>2021</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr"/>
       <c r="Q54" s="4" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
       <c r="S54" s="4" t="inlineStr"/>
       <c r="T54" s="4" t="inlineStr">
         <is>
@@ -9284,35 +8550,21 @@
         </is>
       </c>
       <c r="U54" s="4" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
       <c r="W54" s="4" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
       <c r="Y54" s="4" t="inlineStr"/>
-      <c r="Z54" t="inlineStr"/>
-      <c r="AA54" t="inlineStr"/>
-      <c r="AB54" t="inlineStr"/>
       <c r="AC54" s="4" t="inlineStr"/>
-      <c r="AD54" t="inlineStr"/>
       <c r="AE54" s="4" t="inlineStr"/>
       <c r="AF54" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG54" t="inlineStr"/>
-      <c r="AH54" t="inlineStr"/>
-      <c r="AI54" t="inlineStr"/>
       <c r="AJ54" s="4" t="inlineStr"/>
-      <c r="AK54" t="inlineStr"/>
       <c r="AL54" s="4" t="inlineStr"/>
       <c r="AM54" s="4" t="inlineStr"/>
       <c r="AN54" s="4" t="inlineStr"/>
       <c r="AO54" s="4" t="inlineStr"/>
-      <c r="AP54" t="inlineStr"/>
-      <c r="AQ54" t="inlineStr"/>
-      <c r="AR54" t="inlineStr"/>
       <c r="AS54" s="4" t="inlineStr"/>
-      <c r="AT54" t="inlineStr"/>
       <c r="AU54" t="inlineStr">
         <is>
           <t>T100000130354</t>
@@ -9334,7 +8586,7 @@
       <c r="BA54" s="4" t="inlineStr"/>
       <c r="BB54" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Goldboro_LNG_Terminal</t>
+          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Goldboro_LNG_Terminal | CBC, https://www.cbc.ca/news/canada/nova-scotia/proposed-goldboro-lng-plant-abandoned-after-11-years-1.7038936 | GEM, https://www.gem.wiki/Goldboro_LNG_Terminal</t>
         </is>
       </c>
     </row>
@@ -9349,8 +8601,6 @@
           <t>Nisga'a LNG Terminal</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" s="11" t="inlineStr">
         <is>
           <t>inactive</t>
@@ -9376,7 +8626,6 @@
           <t>Portland Inlet</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" s="4" t="inlineStr">
         <is>
           <t>Government of Nisga’a Lisims [100.0%]</t>
@@ -9392,11 +8641,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
       <c r="Q55" s="4" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
       <c r="S55" s="4" t="inlineStr"/>
       <c r="T55" s="4" t="inlineStr">
         <is>
@@ -9404,35 +8649,21 @@
         </is>
       </c>
       <c r="U55" s="4" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
       <c r="W55" s="4" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
       <c r="Y55" s="4" t="inlineStr"/>
-      <c r="Z55" t="inlineStr"/>
-      <c r="AA55" t="inlineStr"/>
-      <c r="AB55" t="inlineStr"/>
       <c r="AC55" s="4" t="inlineStr"/>
-      <c r="AD55" t="inlineStr"/>
       <c r="AE55" s="4" t="inlineStr"/>
       <c r="AF55" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG55" t="inlineStr"/>
-      <c r="AH55" t="inlineStr"/>
-      <c r="AI55" t="inlineStr"/>
       <c r="AJ55" s="4" t="inlineStr"/>
-      <c r="AK55" t="inlineStr"/>
       <c r="AL55" s="4" t="inlineStr"/>
       <c r="AM55" s="4" t="inlineStr"/>
       <c r="AN55" s="4" t="inlineStr"/>
       <c r="AO55" s="4" t="inlineStr"/>
-      <c r="AP55" t="inlineStr"/>
-      <c r="AQ55" t="inlineStr"/>
-      <c r="AR55" t="inlineStr"/>
       <c r="AS55" s="4" t="inlineStr"/>
-      <c r="AT55" t="inlineStr"/>
       <c r="AU55" t="inlineStr">
         <is>
           <t>T100000130361</t>
@@ -9504,7 +8735,6 @@
           <t>Saint John</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" s="4" t="inlineStr">
         <is>
           <t>Repsol SA [100.0%]</t>
@@ -9520,11 +8750,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
       <c r="Q56" s="4" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
       <c r="S56" s="4" t="inlineStr"/>
       <c r="T56" s="4" t="inlineStr">
         <is>
@@ -9532,7 +8758,6 @@
         </is>
       </c>
       <c r="U56" s="4" t="inlineStr"/>
-      <c r="V56" t="inlineStr"/>
       <c r="W56" s="4" t="inlineStr"/>
       <c r="X56" t="inlineStr">
         <is>
@@ -9547,30 +8772,19 @@
       <c r="Z56" t="n">
         <v>3050</v>
       </c>
-      <c r="AA56" t="inlineStr"/>
-      <c r="AB56" t="inlineStr"/>
       <c r="AC56" s="4" t="inlineStr"/>
-      <c r="AD56" t="inlineStr"/>
       <c r="AE56" s="4" t="inlineStr"/>
       <c r="AF56" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="AG56" t="inlineStr"/>
-      <c r="AH56" t="inlineStr"/>
-      <c r="AI56" t="inlineStr"/>
       <c r="AJ56" s="4" t="inlineStr"/>
-      <c r="AK56" t="inlineStr"/>
       <c r="AL56" s="4" t="inlineStr"/>
       <c r="AM56" s="4" t="inlineStr"/>
       <c r="AN56" s="4" t="inlineStr"/>
       <c r="AO56" s="4" t="inlineStr"/>
-      <c r="AP56" t="inlineStr"/>
-      <c r="AQ56" t="inlineStr"/>
-      <c r="AR56" t="inlineStr"/>
       <c r="AS56" s="4" t="inlineStr"/>
-      <c r="AT56" t="inlineStr"/>
       <c r="AU56" t="inlineStr">
         <is>
           <t>T100000130349</t>
@@ -9593,6 +8807,158 @@
       <c r="BB56" s="4" t="inlineStr">
         <is>
           <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Saint_John_LNG_Terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>kanata_lng</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Kanata LNG</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>early_proposed</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Announced 16 June 2026 via a non-binding memorandum of understanding between Kanata Clean Power and Hanwha Ocean. Estimated capital cost US$15.7 billion. No regulatory filing has been made and the gas transport route is described only as being from northeast British Columbia by unspecified means.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>British Columbia</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>Prince Rupert, British Columbia</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Kanata Clean Power &amp; Climate Technologies Corp.</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>Kanata Clean Power; Hanwha Ocean (non-binding MOU); up to 50% offered to participating First Nations</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="4" t="n"/>
+      <c r="R57" t="n">
+        <v>12</v>
+      </c>
+      <c r="S57" s="4" t="inlineStr">
+        <is>
+          <t>Up to 12 mtpa as stated by the proponent. No filed project description or environmental assessment.</t>
+        </is>
+      </c>
+      <c r="T57" s="4" t="inlineStr">
+        <is>
+          <t>overseas export</t>
+        </is>
+      </c>
+      <c r="U57" s="4" t="n"/>
+      <c r="V57" t="n">
+        <v>0</v>
+      </c>
+      <c r="W57" s="4" t="inlineStr">
+        <is>
+          <t>Export project.</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="Y57" s="4" t="n"/>
+      <c r="AC57" s="4" t="n"/>
+      <c r="AE57" s="4" t="inlineStr">
+        <is>
+          <t>The Prince Rupert Port Authority stated it had no awareness of the project and that no LNG developments were being considered on lands within its jurisdiction. Kanata says governments and rights-holding First Nations were given advance notice, and Gitxaala Enterprises Corporation has confirmed early talks, but the company has declined to name other parties.</t>
+        </is>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>export, floating</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="AI57" t="inlineStr">
+        <is>
+          <t>gas_turbine</t>
+        </is>
+      </c>
+      <c r="AJ57" s="4" t="inlineStr">
+        <is>
+          <t>previously classified as not_published.</t>
+        </is>
+      </c>
+      <c r="AK57" t="inlineStr">
+        <is>
+          <t>export</t>
+        </is>
+      </c>
+      <c r="AL57" s="4" t="inlineStr">
+        <is>
+          <t>Assigned from end_use. Recorded explicitly so chain selection is a decision in the register rather than a text match on free text.</t>
+        </is>
+      </c>
+      <c r="AM57" s="4" t="n"/>
+      <c r="AN57" s="4" t="n"/>
+      <c r="AO57" s="4" t="n"/>
+      <c r="AS57" s="4" t="inlineStr">
+        <is>
+          <t>No export licence. Has not applied.</t>
+        </is>
+      </c>
+      <c r="AV57" s="4" t="n"/>
+      <c r="AW57" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AX57" s="4" t="n"/>
+      <c r="AY57" s="4" t="inlineStr">
+        <is>
+          <t>None. Has not applied.</t>
+        </is>
+      </c>
+      <c r="AZ57" s="4" t="n"/>
+      <c r="BA57" s="4" t="n"/>
+      <c r="BB57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html | Energy Intelligence, 18 June 2026, https://www.energyintel.com/0000019e-d707-d1c7-a9bf-ff5fb8d50000</t>
         </is>
       </c>
     </row>
@@ -9608,7 +8974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB56"/>
+  <dimension ref="A1:BB57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -10394,7 +9760,7 @@
       </c>
       <c r="AK3" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source and electrification_commitment in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL3" s="4" t="inlineStr">
@@ -12026,7 +11392,7 @@
       </c>
       <c r="AK9" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source and electrification_commitment in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL9" s="4" t="inlineStr">
@@ -12298,7 +11664,7 @@
       </c>
       <c r="AK10" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source and electrification_commitment in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL10" s="4" t="inlineStr">
@@ -12570,7 +11936,7 @@
       </c>
       <c r="AK11" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source and electrification_commitment in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL11" s="4" t="inlineStr">
@@ -12842,7 +12208,7 @@
       </c>
       <c r="AK12" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source and electrification_commitment in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL12" s="4" t="inlineStr">
@@ -13114,7 +12480,7 @@
       </c>
       <c r="AK13" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source and electrification_commitment in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL13" s="4" t="inlineStr">
@@ -13386,7 +12752,7 @@
       </c>
       <c r="AK14" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source and electrification_commitment in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL14" s="4" t="inlineStr">
@@ -13930,7 +13296,7 @@
       </c>
       <c r="AK16" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL16" s="4" t="inlineStr">
@@ -14202,7 +13568,7 @@
       </c>
       <c r="AK17" s="4" t="inlineStr">
         <is>
-          <t>Derived from power_source in this register</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL17" s="4" t="inlineStr">
@@ -14329,17 +13695,17 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ State/Province</t>
+          <t>GEM wiki: https://www.gem.wiki/Fermeuse_Energy_FLNG_Terminal</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ Location</t>
+          <t>CBC, 10 February 2026, https://www.cbc.ca/news/canada/newfoundland-labrador/fermeuse-lng-proposed-project-9.7082941 | GEM wiki: https://www.gem.wiki/Fermeuse_Energy_FLNG_Terminal</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Fermeuse Energy news release, 2 September 2025</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
@@ -14379,12 +13745,12 @@
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Derived from proponent-stated 9.7 Tcf Jeanne d'Arc reserve over 40 years; not a published nameplate</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/</t>
+          <t>Compiled by us; derivation recorded in capacity_basis</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -14444,12 +13810,12 @@
       </c>
       <c r="AE18" s="4" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Fermeuse Energy news release, 2 September 2025 | CBC, 10 February 2026, https://www.cbc.ca/news/canada/newfoundland-labrador/fermeuse-lng-proposed-project-9.7082941</t>
         </is>
       </c>
       <c r="AF18" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ FacilityType</t>
+          <t>GEM wiki: https://www.gem.wiki/Fermeuse_Energy_FLNG_Terminal</t>
         </is>
       </c>
       <c r="AG18" s="4" t="inlineStr">
@@ -14469,17 +13835,17 @@
       </c>
       <c r="AJ18" s="4" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Compiled by us</t>
         </is>
       </c>
       <c r="AK18" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL18" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Compiled by us</t>
         </is>
       </c>
       <c r="AM18" s="4" t="inlineStr">
@@ -15946,17 +15312,17 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Assigned by us from status, regulatory stage and FID - see tier_reason</t>
+          <t>Assigned by us - see tier_reason</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Derived: advanced_proposed and early_proposed group as proposed</t>
+          <t>Assigned: proposed</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Discovery_LNG_Terminal</t>
+          <t>Compiled by us; August 2026 news and regulatory review found no current filing</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -15966,12 +15332,12 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ Location</t>
+          <t>GEM GGIT LNG Terminals (Sep 2025) Location; province appended</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Compiled by us from review of news and regulatory sources, August 2026</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -15981,7 +15347,7 @@
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ Status</t>
+          <t>Assigned: proposed, pending verification August 2026</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
@@ -16001,7 +15367,7 @@
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ ActualStartYear or LatestPlannedStartYear</t>
+          <t>Not available</t>
         </is>
       </c>
       <c r="Q24" s="4" t="inlineStr">
@@ -16076,7 +15442,7 @@
       </c>
       <c r="AE24" s="4" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Compiled by us</t>
         </is>
       </c>
       <c r="AF24" s="4" t="inlineStr">
@@ -16096,22 +15462,22 @@
       </c>
       <c r="AI24" s="4" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Assigned by us from end_use</t>
         </is>
       </c>
       <c r="AJ24" s="4" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Compiled by us</t>
         </is>
       </c>
       <c r="AK24" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
         </is>
       </c>
       <c r="AL24" s="4" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>Compiled by us</t>
         </is>
       </c>
       <c r="AM24" s="4" t="inlineStr">
@@ -17316,7 +16682,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Grassy_Point_LNG_Terminal</t>
+          <t>IAAC registry, https://iaac-aeic.gc.ca/050/evaluations/proj/80089</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -18132,7 +17498,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Bear_Head_LNG_Terminal</t>
+          <t>Nova Scotia EA registry, https://novascotia.ca/nse/ea/bear-head-energy/ | Bear Head Energy, https://www.bearheadenergy.ca/our-project</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -19492,7 +18858,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Grassy_Point_LNG_Terminal</t>
+          <t>IAAC registry, https://iaac-aeic.gc.ca/050/evaluations/proj/80089</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -23844,7 +23210,7 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Goldboro_LNG_Terminal</t>
+          <t>CBC, https://www.cbc.ca/news/canada/nova-scotia/proposed-goldboro-lng-plant-abandoned-after-11-years-1.7038936 | GEM, https://www.gem.wiki/Goldboro_LNG_Terminal</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -23869,7 +23235,7 @@
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ Status</t>
+          <t>CBC, https://www.cbc.ca/news/canada/nova-scotia/proposed-goldboro-lng-plant-abandoned-after-11-years-1.7038936 | GEM, https://www.gem.wiki/Goldboro_LNG_Terminal</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -24116,7 +23482,7 @@
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ | GEM wiki: https://www.gem.wiki/Goldboro_LNG_Terminal</t>
+          <t>CBC, https://www.cbc.ca/news/canada/nova-scotia/proposed-goldboro-lng-plant-abandoned-after-11-years-1.7038936 | GEM, https://www.gem.wiki/Goldboro_LNG_Terminal</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -24141,7 +23507,7 @@
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>GEM GGIT LNG Terminals (Sep 2025): https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/ Status</t>
+          <t>CBC, https://www.cbc.ca/news/canada/nova-scotia/proposed-goldboro-lng-plant-abandoned-after-11-years-1.7038936 | GEM, https://www.gem.wiki/Goldboro_LNG_Terminal</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -24894,6 +24260,278 @@
         </is>
       </c>
       <c r="BB56" s="4" t="inlineStr">
+        <is>
+          <t>Compiled by us from the sources named in this row</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>kanata_lng</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Kanata LNG</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Assigned by us - see tier_reason</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Assigned: proposed</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>Energy Intelligence, 18 June 2026, https://www.energyintel.com/0000019e-d707-d1c7-a9bf-ff5fb8d50000</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html | Energy Intelligence, 18 June 2026, https://www.energyintel.com/0000019e-d707-d1c7-a9bf-ff5fb8d50000</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>Date we last verified against the sources listed</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="P57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Q57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="R57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="S57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="T57" s="4" t="inlineStr">
+        <is>
+          <t>Derived: classified as an export project</t>
+        </is>
+      </c>
+      <c r="U57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="V57" s="4" t="inlineStr">
+        <is>
+          <t>Derived: export projects supply no LNG to the domestic market</t>
+        </is>
+      </c>
+      <c r="W57" s="4" t="inlineStr">
+        <is>
+          <t>Compiled by us</t>
+        </is>
+      </c>
+      <c r="X57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Y57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="Z57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AA57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AB57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AC57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AD57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AE57" s="4" t="inlineStr">
+        <is>
+          <t>Energy Intelligence, 18 June 2026, https://www.energyintel.com/0000019e-d707-d1c7-a9bf-ff5fb8d50000</t>
+        </is>
+      </c>
+      <c r="AF57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="AG57" s="4" t="inlineStr">
+        <is>
+          <t>Hanwha Ocean news release, 16 June 2026, https://www.newswire.ca/news-releases/hanwha-ocean-signs-strategic-memorandum-of-understanding-with-kanata-clean-power-for-proposed-floating-lng-project-in-canada-867061587.html</t>
+        </is>
+      </c>
+      <c r="AH57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AI57" s="4" t="inlineStr">
+        <is>
+          <t>Assigned by us from end_use</t>
+        </is>
+      </c>
+      <c r="AJ57" s="4" t="inlineStr">
+        <is>
+          <t>Compiled by us</t>
+        </is>
+      </c>
+      <c r="AK57" s="4" t="inlineStr">
+        <is>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
+        </is>
+      </c>
+      <c r="AL57" s="4" t="inlineStr">
+        <is>
+          <t>Compiled by us</t>
+        </is>
+      </c>
+      <c r="AM57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AN57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AO57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AP57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AQ57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AR57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AS57" s="4" t="inlineStr">
+        <is>
+          <t>CER Export Licence Applications schedule</t>
+        </is>
+      </c>
+      <c r="AT57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AU57" s="4" t="inlineStr">
+        <is>
+          <t>Not available - project does not appear in GEM GGIT LNG Terminals Sep 2025</t>
+        </is>
+      </c>
+      <c r="AV57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AW57" s="4" t="inlineStr">
+        <is>
+          <t>NRCan Canadian LNG projects: not present as of August 2026</t>
+        </is>
+      </c>
+      <c r="AX57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AY57" s="4" t="inlineStr">
+        <is>
+          <t>CER Export Licence Applications schedule</t>
+        </is>
+      </c>
+      <c r="AZ57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="BA57" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="BB57" s="4" t="inlineStr">
         <is>
           <t>Compiled by us from the sources named in this row</t>
         </is>
@@ -25108,8 +24746,6 @@
       <c r="E3" t="n">
         <v>21.46</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
         <is>
           <t>LNG Canada Terminal</t>
@@ -25251,8 +24887,6 @@
         <v>2028</v>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
         <v>4.09</v>
       </c>
@@ -25379,10 +25013,7 @@
       <c r="F7" t="n">
         <v>471</v>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
         <v>13.9</v>
       </c>
@@ -26871,7 +26502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -26927,22 +26558,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Blank</t>
+          <t>Derived 5.0 mtpa</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>No capacity disclosed by proponent or GEM</t>
+          <t>Proponent has not published a liquefaction capacity. 5.0 mtpa is the lowest defensible derivation from the stated 9.7 Tcf Jeanne d'Arc reserve over a 40-year life at 1.38 bcm per mtpa. Higher figures (8.0 from a 25-year life; 9–12 from capital-cost benchmarking; an unsourced 10 mtpa) were not used.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Company filing once an LNG plant proposal is submitted</t>
+          <t>A filed project description stating liquefaction capacity.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>high - would change totals if the project advances</t>
+          <t>high - derived figure now enters totals; replace when a published capacity exists</t>
         </is>
       </c>
     </row>
@@ -27551,6 +27182,38 @@
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>high - central to the electrification rebuttal</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Discovery LNG Terminal</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Least verified asset in the register</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Moved from inactive to early_proposed pending verification. Capacity is the GEM nameplate of 20 mtpa. No current filing or proponent activity was located in a review of news and regulatory sources in August 2026.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>A current regulatory filing, proponent update, or confirmation the proposal is dead.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>high - 20 mtpa early_proposed; classification should be revisited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Kino Aski to 15 mtpa and publish electrification appendix and slide tables.
Headline is now 272.0 Mt/yr at 100.1 mtpa export so teammates clone a complete, validated run.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Asset_Register.xlsx
+++ b/Inputs/Canada_LNG_Asset_Register.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>All Canadian LNG terminals in GEM GGIT (Sep 2025), plus projects not in GEM found by research: Summit Lake PG LNG, Marinvest Baie-Comeau, the Tilbury Marine Jetty, and Kanata LNG. Discovery LNG is in GEM but was moved from inactive to early_proposed pending verification.</t>
+          <t>All Canadian LNG terminals in GEM GGIT (Sep 2025), plus projects not in GEM found by research: Summit Lake PG LNG, Kino Aski LNG (formerly Marinvest Baie-Comeau), the Tilbury Marine Jetty, and Kanata LNG. Discovery LNG is in GEM but was moved from inactive to early_proposed pending verification.</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Announced, but no completed regulatory filing. Groups with advanced_proposed as proposed in the calculation, but the tier is retained so the difference in maturity stays visible. Capacity figures here are weaker: Baie-Comeau's 10 mtpa is a company statement to journalists and Summit Lake's 2.7 is an upper bound from a suspended assessment.</t>
+          <t>Announced, but no completed regulatory filing. Groups with advanced_proposed as proposed in the calculation, but the tier is retained so the difference in maturity stays visible. Capacity figures here are weaker: Kino Aski's 15 mtpa is a proponent press release, not a filed figure, and Summit Lake's 2.7 is an upper bound from a suspended assessment.</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Baie-Comeau's 10 mtpa is a company statement to journalists rather than a filed figure. Summit Lake's 2.7 is an upper bound from its impact assessment. Both are flagged in capacity_basis.</t>
+          <t>Kino Aski's 15 mtpa is from the proponent's 17 August 2026 press release rather than a filed project description; the earlier 10 mtpa journalist statement is replaced. The feedgas pipeline route is undefined. Summit Lake's 2.7 is an upper bound from its impact assessment. Both are flagged in capacity_basis.</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Marinvest Energy LNG Export Project (Baie-Comeau)</t>
+          <t>Kino Aski LNG (formerly Marinvest Energy, Baie-Comeau)</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>No initial project description filed with the Impact Assessment Agency as of early 2026, despite federal facilitation.</t>
+          <t>Early-stage proposal. The 17 August 2026 release states that no formal regulatory process has yet begun. No initial project description has been filed with the Impact Assessment Agency. The feedgas pipeline from Western Canada is described only as a combination of existing and new infrastructure; the route is undefined.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -3929,12 +3929,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Marinvest Energy Canada</t>
+          <t>Kino Aski Inc.; Marinvest Energy Canada Inc.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Marinvest Energy AS (Norway)</t>
+          <t>Kino Aski Inc. majority, Atikamekw Nation-led; Marinvest Energy Canada Inc. minority</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N16" t="b">
@@ -3952,11 +3952,11 @@
       </c>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>company statement to journalists; not a filed figure</t>
+          <t>Proponent press release, 17 August 2026: up to 15 mtpa. Replaces the earlier 10 mtpa figure, which was a company statement to journalists rather than a filed or released capacity.</t>
         </is>
       </c>
       <c r="T16" s="4" t="inlineStr">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="Y16" s="4" t="inlineStr">
         <is>
-          <t>Baie-Comeau, St Lawrence River, marine to northwest Europe</t>
+          <t>Baie-Comeau, St Lawrence River, marine to northwest Europe. Feedgas from Western Canada by unspecified existing and new pipelines; route undefined.</t>
         </is>
       </c>
       <c r="Z16" t="n">
@@ -3989,7 +3989,7 @@
       <c r="AC16" s="4" t="inlineStr"/>
       <c r="AE16" s="4" t="inlineStr">
         <is>
-          <t>Route distance not sourced</t>
+          <t>No regulatory process has begun. The pipeline route from Western Canada to Baie-Comeau is undefined. The release claims renewable electricity in Quebec; electric drive is not assumed.</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="AM16" s="4" t="inlineStr">
         <is>
-          <t>Company reported to be planning its own wind farm to supply the plant</t>
+          <t>Proponent states the plant would be powered by renewable electricity in Quebec. No contracted supply or interconnection identified.</t>
         </is>
       </c>
       <c r="AN16" s="4" t="inlineStr">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="AO16" s="4" t="inlineStr">
         <is>
-          <t>Aspirational - no filed plan</t>
+          <t>Aspirational - 17 August 2026 release claims renewable power; no contracted supply. Electric drive is not assumed.</t>
         </is>
       </c>
       <c r="AS16" s="4" t="inlineStr">
@@ -4065,7 +4065,7 @@
       <c r="BA16" s="4" t="inlineStr"/>
       <c r="BB16" s="4" t="inlineStr">
         <is>
-          <t>The Narwhal, Baie-Comeau LNG explained: https://thenarwhal.ca/lng-export-project-baie-comeau-quebec/ | Greenpeace Canada, Marinvest: https://www.greenpeace.org/canada/en/story/75493/marinvest-the-biggest-lng-project-youve-never-heard-of/ | CBC: https://www.cbc.ca/news/canada/montreal/quebec-lng-baie-comeau-1.7648993 | National Observer: https://www.nationalobserver.com/2026/02/20/news/marinvest-quebec-lng-project-ottawa</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html | The Narwhal, Baie-Comeau LNG explained: https://thenarwhal.ca/lng-export-project-baie-comeau-quebec/ | Greenpeace Canada, Marinvest: https://www.greenpeace.org/canada/en/story/75493/marinvest-the-biggest-lng-project-youve-never-heard-of/ | CBC: https://www.cbc.ca/news/canada/montreal/quebec-lng-baie-comeau-1.7648993 | National Observer: https://www.nationalobserver.com/2026/02/20/news/marinvest-quebec-lng-project-ottawa</t>
         </is>
       </c>
     </row>
@@ -13121,7 +13121,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Marinvest Energy LNG Export Project (Baie-Comeau)</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>The Narwhal, Baie-Comeau LNG explained: https://thenarwhal.ca/lng-export-project-baie-comeau-quebec/</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -13161,12 +13161,12 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>The Narwhal, Baie-Comeau LNG explained: https://thenarwhal.ca/lng-export-project-baie-comeau-quebec/ - Marinvest Energy Canada, subsidiary of Marinvest Energy AS (Norway)</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>The Narwhal, Baie-Comeau LNG explained: https://thenarwhal.ca/lng-export-project-baie-comeau-quebec/ - Marinvest Energy Canada, subsidiary of Marinvest Energy AS (Norway)</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -13201,12 +13201,12 @@
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>Greenpeace Canada, Marinvest: https://www.greenpeace.org/canada/en/story/75493/marinvest-the-biggest-lng-project-youve-never-heard-of/ - company stated 10 mtpa under questioning; corroborated by The Narwhal, Baie-Comeau LNG explained: https://thenarwhal.ca/lng-export-project-baie-comeau-quebec/</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>Greenpeace Canada, Marinvest: https://www.greenpeace.org/canada/en/story/75493/marinvest-the-biggest-lng-project-youve-never-heard-of/ - company stated 10 mtpa under questioning; corroborated by The Narwhal, Baie-Comeau LNG explained: https://thenarwhal.ca/lng-export-project-baie-comeau-quebec/</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="T16" s="4" t="inlineStr">
@@ -13236,7 +13236,7 @@
       </c>
       <c r="Y16" s="4" t="inlineStr">
         <is>
-          <t>Proponent statements - see sources column</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="Z16" s="4" t="inlineStr">
@@ -13266,47 +13266,47 @@
       </c>
       <c r="AE16" s="4" t="inlineStr">
         <is>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
+        </is>
+      </c>
+      <c r="AF16" s="4" t="inlineStr">
+        <is>
+          <t>Derived: export project</t>
+        </is>
+      </c>
+      <c r="AG16" s="4" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="AH16" s="4" t="inlineStr">
+        <is>
+          <t>National Observer: https://www.nationalobserver.com/2026/02/20/news/marinvest-quebec-lng-project-ottawa</t>
+        </is>
+      </c>
+      <c r="AI16" s="4" t="inlineStr">
+        <is>
+          <t>Assigned by us from end_use</t>
+        </is>
+      </c>
+      <c r="AJ16" s="4" t="inlineStr">
+        <is>
           <t>Compiled by us</t>
         </is>
       </c>
-      <c r="AF16" s="4" t="inlineStr">
-        <is>
-          <t>Derived: export project</t>
-        </is>
-      </c>
-      <c r="AG16" s="4" t="inlineStr">
-        <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="AH16" s="4" t="inlineStr">
+      <c r="AK16" s="4" t="inlineStr">
+        <is>
+          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
+        </is>
+      </c>
+      <c r="AL16" s="4" t="inlineStr">
         <is>
           <t>National Observer: https://www.nationalobserver.com/2026/02/20/news/marinvest-quebec-lng-project-ottawa</t>
         </is>
       </c>
-      <c r="AI16" s="4" t="inlineStr">
-        <is>
-          <t>Assigned by us from end_use</t>
-        </is>
-      </c>
-      <c r="AJ16" s="4" t="inlineStr">
-        <is>
-          <t>Compiled by us</t>
-        </is>
-      </c>
-      <c r="AK16" s="4" t="inlineStr">
-        <is>
-          <t>Assigned gas_turbine, August 2026 electrification revision; previous classification retained in liquefaction_drive_note</t>
-        </is>
-      </c>
-      <c r="AL16" s="4" t="inlineStr">
-        <is>
-          <t>National Observer: https://www.nationalobserver.com/2026/02/20/news/marinvest-quebec-lng-project-ottawa</t>
-        </is>
-      </c>
       <c r="AM16" s="4" t="inlineStr">
         <is>
-          <t>National Observer: https://www.nationalobserver.com/2026/02/20/news/marinvest-quebec-lng-project-ottawa</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="AN16" s="4" t="inlineStr">
@@ -13316,7 +13316,7 @@
       </c>
       <c r="AO16" s="4" t="inlineStr">
         <is>
-          <t>National Observer: https://www.nationalobserver.com/2026/02/20/news/marinvest-quebec-lng-project-ottawa</t>
+          <t>Kino Aski Inc. news release, 17 August 2026, https://www.newswire.ca/news-releases/first-nations-lead-kino-aski-lng-a-major-canadian-energy-project-800865754.html</t>
         </is>
       </c>
       <c r="AP16" s="4" t="inlineStr">
@@ -26777,22 +26777,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Baie-Comeau and Summit Lake</t>
+          <t>Kino Aski LNG (Baie-Comeau) and Summit Lake</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Weaker basis</t>
+          <t>Press release / weaker basis</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Baie-Comeau 10 mtpa is a company statement to journalists, not a filed figure. Summit Lake 2.7 mtpa is an 'up to' design maximum.</t>
+          <t>Kino Aski's 15 mtpa is from the proponent's 17 August 2026 press release; no project description has been filed and no regulatory process has begun. Summit Lake 2.7 mtpa remains an 'up to' design maximum from a suspended assessment.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Filed project descriptions once submitted</t>
+          <t>Filed project descriptions once submitted; a defined feedgas pipeline route for Kino Aski.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -27065,7 +27065,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Summit Lake, Baie-Comeau</t>
+          <t>Summit Lake, Kino Aski LNG (Baie-Comeau)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">

</xml_diff>

<commit_message>
Re-derive upstream on pipeline 0.074, net Fermeuse liquefaction fuel, and lock 7,167.1 Mt.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Asset_Register.xlsx
+++ b/Inputs/Canada_LNG_Asset_Register.xlsx
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Fermeuse Energy has not published a liquefaction capacity. The register records 5.0 mtpa, the lowest defensible derivation from the stated 9.7 Tcf Jeanne d'Arc reserve over a 40-year life. This is an exception to the nameplate convention and is flagged in capacity_basis.</t>
+          <t>Fermeuse Energy has not published a liquefaction capacity. The register records 4.5 mtpa, derived from the stated 9.7 Tcf Jeanne d'Arc resource over a 40-year life, net of the gas liquefaction burns as fuel. The derivation is conditional on the proponent's resource claim and assumes full recovery on a flat profile, both of which push it up; it is not a lower bound. This is an exception to the nameplate convention and is flagged in capacity_basis.</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       <c r="AC17" s="4" t="inlineStr"/>
       <c r="AE17" s="4" t="inlineStr">
         <is>
-          <t>Rail leg has no analogue in the other projects and is not yet modelled</t>
+          <t>Rail leg has no analogue in the other projects and is not modelled. SHIPPING MODE: the proponent's concept is LNG in ISO containers railed to Prince Rupert and shipped in container vessels, not LNG carriers. The model applies the LNG-carrier shipping factor (0.12 tCO2e/t on the 3,800 nm basis) to this asset like every other export terminal. At 2.7 mtpa the shipping stage is about 0.3 MtCO2e/yr, so any difference between containerised and carrier shipping intensity is immaterial to every published figure; recorded 3 September 2026 so the substitution is visible rather than silent.</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4458,11 +4458,11 @@
       </c>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>Derived, not published. The proponent has not stated a liquefaction capacity. This figure is constrained by the gas resource: Fermeuse Energy states the project would develop 9.7 trillion cubic feet of offshore associated gas in the Jeanne d'Arc Basin, which is 275 billion cubic metres. At 1.38 bcm per mtpa, spread over the 40-year operating life assumed elsewhere in this register, that supports 5.0 mtpa. Two other approaches give higher figures and were not used: the same reserve over a 25-year life gives 8.0 mtpa, and benchmarking the stated US$12 to 15 billion capital cost against Ksi Lisims and Cedar gives 9 to 12 mtpa. An unsourced third-party table circulates a figure of 10 mtpa. The lowest defensible derivation is used.</t>
+          <t>Derived, not published, and conditional on the proponent's own resource claim. The proponent has not stated a liquefaction capacity. Fermeuse Energy states the project would develop 9.7 trillion cubic feet of offshore associated gas in the Jeanne d'Arc Basin, which is 275 billion cubic metres. DERIVATION: 275 bcm / 1.38 bcm per mtpa (lng_to_gas_bcm_per_mtpa, the gas-equivalent of LNG OUTPUT) / 40 years = 4.98 mtpa of output if every molecule became LNG. It does not: liquefaction burns part of the throughput as fuel. Using the model's own factors so the derivation is internally consistent, the liquefaction stage emits 0.29 tCO2e per t LNG and burning gas releases 2.75 tCO2 per t (combustion central), so fuel is 0.29 / 2.75 = 0.1055 t per t LNG and feedgas per tonne of LNG is 1.1055 t. Output is therefore 4.98 / 1.1055 = 4.51, recorded as 4.5 mtpa. That treats the whole liquefaction factor as fuel combustion; the small non-combustion part (flaring, venting) makes the fuel share slightly high and the capacity slightly low, inside the rounding. WHAT PUSHES THIS FIGURE UP, and why it is not a lower bound: it assumes (a) 100 per cent recovery of a resource stated by the proponent, not a regulator or an independent estimate; (b) a flat 40-year production profile, whereas associated gas follows the oil decline and would front-load output; and (c) no reservation of gas for platform fuel, reinjection or domestic supply. Each choice raises the capacity, so the figure is closer to an upper bound on the proponent's claim than to a conservative one. Two other approaches give higher figures and were not used: the same resource over a 25-year life gives about 8 mtpa net of fuel, and benchmarking the stated US$12 to 15 billion capital cost against Ksi Lisims and Cedar gives 9 to 12 mtpa. An unsourced third-party table circulates a figure of 10 mtpa. HISTORY: 5.0 mtpa until 3 September 2026, from the same resource without netting the fuel share, and described as 'the lowest defensible derivation', which it was not.</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -14054,7 +14054,7 @@
       </c>
       <c r="AE17" s="4" t="inlineStr">
         <is>
-          <t>Compiled by us</t>
+          <t>Compiled by us; shipping mode from the export_route already sourced in this row (BC EAO project description)</t>
         </is>
       </c>
       <c r="AF17" s="4" t="inlineStr">
@@ -14281,12 +14281,12 @@
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>Derived from proponent-stated 9.7 Tcf Jeanne d'Arc reserve over 40 years; not a published nameplate</t>
+          <t>Derived from proponent-stated 9.7 Tcf Jeanne d'Arc resource over 40 years, net of liquefaction fuel at the model's own liquefaction and combustion factors; not a published nameplate. Fermeuse Energy news release, 2 September 2025.</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>Compiled by us; derivation recorded in capacity_basis</t>
+          <t>Compiled by us; derivation recorded step by step in capacity_basis</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -28002,12 +28002,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Derived 5.0 mtpa</t>
+          <t>Derived 4.5 mtpa</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Proponent has not published a liquefaction capacity. 5.0 mtpa is the lowest defensible derivation from the stated 9.7 Tcf Jeanne d'Arc reserve over a 40-year life at 1.38 bcm per mtpa. Higher figures (8.0 from a 25-year life; 9–12 from capital-cost benchmarking; an unsourced 10 mtpa) were not used.</t>
+          <t>Proponent has not published a liquefaction capacity. 4.5 mtpa is derived from the stated 9.7 Tcf Jeanne d'Arc resource over a 40-year life at 1.38 bcm per mtpa, net of liquefaction fuel at the model's own factors (was 5.0 before netting fuel, 3 September 2026). Conditional on the proponent's resource claim; full recovery on a flat profile pushes it up. Higher figures (about 8 from a 25-year life; 9-12 from capital-cost benchmarking; an unsourced 10 mtpa) were not used.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">

</xml_diff>